<commit_message>
feat: atualização dos arquivos de screening de fundos imobiliarios
</commit_message>
<xml_diff>
--- a/ranking_fiis.xlsx
+++ b/ranking_fiis.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N85"/>
+  <dimension ref="A1:N75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -515,22 +515,22 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>7.01</v>
+        <v>7.02</v>
       </c>
       <c r="E2" t="n">
-        <v>15.8</v>
+        <v>15.78</v>
       </c>
       <c r="F2" t="n">
-        <v>20.22</v>
+        <v>18.22</v>
       </c>
       <c r="G2" t="n">
         <v>0.73</v>
       </c>
       <c r="H2" t="n">
-        <v>278729000</v>
+        <v>279126000</v>
       </c>
       <c r="I2" t="n">
-        <v>912260</v>
+        <v>803094</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -539,13 +539,13 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M2" t="n">
         <v>2</v>
       </c>
       <c r="N2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="3">
@@ -554,31 +554,31 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>OUJP11</t>
+          <t>HABT11</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>73.2</v>
+        <v>68.95</v>
       </c>
       <c r="E3" t="n">
-        <v>18.07</v>
+        <v>16.45</v>
       </c>
       <c r="F3" t="n">
-        <v>18.53</v>
+        <v>14.92</v>
       </c>
       <c r="G3" t="n">
-        <v>0.73</v>
+        <v>0.72</v>
       </c>
       <c r="H3" t="n">
-        <v>238075000</v>
+        <v>560342000</v>
       </c>
       <c r="I3" t="n">
-        <v>728835</v>
+        <v>1083720</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -587,13 +587,13 @@
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="N3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="4">
@@ -602,31 +602,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>HABT11</t>
+          <t>RPRI11</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>71.33</v>
+        <v>72.37</v>
       </c>
       <c r="E4" t="n">
-        <v>15.9</v>
+        <v>16.99</v>
       </c>
       <c r="F4" t="n">
-        <v>16.06</v>
+        <v>14.73</v>
       </c>
       <c r="G4" t="n">
-        <v>0.75</v>
+        <v>0.72</v>
       </c>
       <c r="H4" t="n">
-        <v>579683000</v>
+        <v>251249000</v>
       </c>
       <c r="I4" t="n">
-        <v>1108400</v>
+        <v>1244300</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -635,13 +635,13 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="N4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -650,31 +650,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>VGHF11</t>
+          <t>VCJR11</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5.87</v>
+        <v>66.91</v>
       </c>
       <c r="E5" t="n">
-        <v>9.779999999999999</v>
+        <v>15.01</v>
       </c>
       <c r="F5" t="n">
-        <v>14.99</v>
+        <v>14.46</v>
       </c>
       <c r="G5" t="n">
-        <v>0.7</v>
+        <v>0.71</v>
       </c>
       <c r="H5" t="n">
-        <v>966916000</v>
+        <v>985181000</v>
       </c>
       <c r="I5" t="n">
-        <v>2370290</v>
+        <v>2473610</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -686,10 +686,10 @@
         <v>1</v>
       </c>
       <c r="M5" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="N5" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -698,46 +698,46 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>VCJR11</t>
+          <t>IRIM11</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Hedge Fund</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>71.59999999999999</v>
+        <v>63.25</v>
       </c>
       <c r="E6" t="n">
-        <v>14.03</v>
+        <v>4.02</v>
       </c>
       <c r="F6" t="n">
-        <v>15.06</v>
+        <v>13.66</v>
       </c>
       <c r="G6" t="n">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="H6" t="n">
-        <v>1054240000</v>
+        <v>2228040000</v>
       </c>
       <c r="I6" t="n">
-        <v>2291490</v>
+        <v>2787360</v>
       </c>
       <c r="J6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="M6" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N6" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
@@ -746,31 +746,31 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>RPRI11</t>
+          <t>RBRY11</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>77.2</v>
+        <v>82.2</v>
       </c>
       <c r="E7" t="n">
-        <v>15.92</v>
+        <v>13.14</v>
       </c>
       <c r="F7" t="n">
-        <v>15.15</v>
+        <v>15.11</v>
       </c>
       <c r="G7" t="n">
-        <v>0.77</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>268017000</v>
+        <v>1049650000</v>
       </c>
       <c r="I7" t="n">
-        <v>1226800</v>
+        <v>3691250</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -779,13 +779,13 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="M7" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="N7" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8">
@@ -794,31 +794,31 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>IRIM11</t>
+          <t>RBRX11</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Hedge Fund</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>65.3</v>
+        <v>7.38</v>
       </c>
       <c r="E8" t="n">
-        <v>3.9</v>
+        <v>5.91</v>
       </c>
       <c r="F8" t="n">
-        <v>14.57</v>
+        <v>13.11</v>
       </c>
       <c r="G8" t="n">
-        <v>0.78</v>
+        <v>0.76</v>
       </c>
       <c r="H8" t="n">
-        <v>2300250000</v>
+        <v>1080090000</v>
       </c>
       <c r="I8" t="n">
-        <v>2960060</v>
+        <v>2291570</v>
       </c>
       <c r="J8" t="n">
         <v>1</v>
@@ -827,13 +827,13 @@
         <v>0</v>
       </c>
       <c r="L8" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="M8" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="N8" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -842,46 +842,46 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MCRE11</t>
+          <t>RVBI11</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>FoF</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>8.43</v>
+        <v>59.9</v>
       </c>
       <c r="E9" t="n">
-        <v>10.88</v>
+        <v>13.05</v>
       </c>
       <c r="F9" t="n">
-        <v>15.27</v>
+        <v>14.1</v>
       </c>
       <c r="G9" t="n">
-        <v>0.83</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H9" t="n">
-        <v>940779000</v>
+        <v>615533000</v>
       </c>
       <c r="I9" t="n">
-        <v>2642070</v>
+        <v>931734</v>
       </c>
       <c r="J9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>11.63</v>
+        <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="M9" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="N9" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10">
@@ -890,31 +890,31 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PSEC11</t>
+          <t>JSAF11</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Hedge Fund</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>55.33</v>
+        <v>6.86</v>
       </c>
       <c r="E10" t="n">
-        <v>10.65</v>
+        <v>13.68</v>
       </c>
       <c r="F10" t="n">
-        <v>13.9</v>
+        <v>12.76</v>
       </c>
       <c r="G10" t="n">
-        <v>0.75</v>
+        <v>0.74</v>
       </c>
       <c r="H10" t="n">
-        <v>1018040000</v>
+        <v>531810000</v>
       </c>
       <c r="I10" t="n">
-        <v>2785300</v>
+        <v>1510150</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="M10" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="N10" t="n">
         <v>29</v>
@@ -938,31 +938,31 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>RVBI11</t>
+          <t>PCIP11</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>59.9</v>
+        <v>73.76000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>13.05</v>
+        <v>13.47</v>
       </c>
       <c r="F11" t="n">
-        <v>14.1</v>
+        <v>12.81</v>
       </c>
       <c r="G11" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="H11" t="n">
-        <v>615533000</v>
+        <v>1254780000</v>
       </c>
       <c r="I11" t="n">
-        <v>931734</v>
+        <v>3093400</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -971,10 +971,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="M11" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="N11" t="n">
         <v>33</v>
@@ -986,46 +986,46 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>XPIN11</t>
+          <t>ITRI11</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>FoF</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>62.04</v>
+        <v>73.94</v>
       </c>
       <c r="E12" t="n">
-        <v>11.45</v>
+        <v>14.05</v>
       </c>
       <c r="F12" t="n">
-        <v>14.43</v>
+        <v>12.81</v>
       </c>
       <c r="G12" t="n">
-        <v>0.83</v>
+        <v>0.79</v>
       </c>
       <c r="H12" t="n">
-        <v>443612000</v>
+        <v>462125000</v>
       </c>
       <c r="I12" t="n">
-        <v>567579</v>
+        <v>1080600</v>
       </c>
       <c r="J12" t="n">
-        <v>81</v>
+        <v>0</v>
       </c>
       <c r="K12" t="n">
-        <v>6.01</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="M12" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="N12" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13">
@@ -1034,46 +1034,46 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>JSAF11</t>
+          <t>GTWR11</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Escritórios</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>7.23</v>
+        <v>78.56</v>
       </c>
       <c r="E13" t="n">
-        <v>12.98</v>
+        <v>13.69</v>
       </c>
       <c r="F13" t="n">
-        <v>13.48</v>
+        <v>12.33</v>
       </c>
       <c r="G13" t="n">
-        <v>0.78</v>
+        <v>0.77</v>
       </c>
       <c r="H13" t="n">
-        <v>560493000</v>
+        <v>942720000</v>
       </c>
       <c r="I13" t="n">
-        <v>1662040</v>
+        <v>647629</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="M13" t="n">
         <v>30</v>
       </c>
       <c r="N13" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14">
@@ -1082,31 +1082,31 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PCIP11</t>
+          <t>VRTA11</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>76.44</v>
+        <v>69.59999999999999</v>
       </c>
       <c r="E14" t="n">
-        <v>13</v>
+        <v>14.48</v>
       </c>
       <c r="F14" t="n">
-        <v>13.87</v>
+        <v>13.12</v>
       </c>
       <c r="G14" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="H14" t="n">
-        <v>1300370000</v>
+        <v>1085230000</v>
       </c>
       <c r="I14" t="n">
-        <v>3072270</v>
+        <v>2298850</v>
       </c>
       <c r="J14" t="n">
         <v>0</v>
@@ -1115,13 +1115,13 @@
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="M14" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="N14" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15">
@@ -1130,46 +1130,46 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CPTS11</t>
+          <t>TRXF11</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Multicategoria</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>7.41</v>
+        <v>81.91</v>
       </c>
       <c r="E15" t="n">
-        <v>6.31</v>
+        <v>5.18</v>
       </c>
       <c r="F15" t="n">
-        <v>14.08</v>
+        <v>12.99</v>
       </c>
       <c r="G15" t="n">
-        <v>0.84</v>
+        <v>0.83</v>
       </c>
       <c r="H15" t="n">
-        <v>2693560000</v>
+        <v>5113700000</v>
       </c>
       <c r="I15" t="n">
-        <v>7857910</v>
+        <v>23370000</v>
       </c>
       <c r="J15" t="n">
-        <v>0</v>
+        <v>97</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="M15" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="N15" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16">
@@ -1178,46 +1178,46 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>GTWR11</t>
+          <t>HSAF11</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Escritórios</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>80.29000000000001</v>
+        <v>74.89</v>
       </c>
       <c r="E16" t="n">
-        <v>13.39</v>
+        <v>15.02</v>
       </c>
       <c r="F16" t="n">
-        <v>13.31</v>
+        <v>13.61</v>
       </c>
       <c r="G16" t="n">
-        <v>0.79</v>
+        <v>0.84</v>
       </c>
       <c r="H16" t="n">
-        <v>963480000</v>
+        <v>189199000</v>
       </c>
       <c r="I16" t="n">
-        <v>697075</v>
+        <v>517814</v>
       </c>
       <c r="J16" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="M16" t="n">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="N16" t="n">
-        <v>46</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17">
@@ -1226,31 +1226,31 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>RBRY11</t>
+          <t>RZAK11</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>87.45999999999999</v>
+        <v>77.5</v>
       </c>
       <c r="E17" t="n">
-        <v>12.35</v>
+        <v>13.75</v>
       </c>
       <c r="F17" t="n">
-        <v>15.48</v>
+        <v>15.19</v>
       </c>
       <c r="G17" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="H17" t="n">
-        <v>1116820000</v>
+        <v>682611000</v>
       </c>
       <c r="I17" t="n">
-        <v>4560880</v>
+        <v>1377320</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1259,13 +1259,13 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="M17" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="N17" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18">
@@ -1274,43 +1274,43 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>RBRX11</t>
+          <t>MCRE11</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>7.92</v>
+        <v>8.73</v>
       </c>
       <c r="E18" t="n">
-        <v>5.5</v>
+        <v>10.51</v>
       </c>
       <c r="F18" t="n">
-        <v>13.41</v>
+        <v>13.51</v>
       </c>
       <c r="G18" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.86</v>
       </c>
       <c r="H18" t="n">
-        <v>1159130000</v>
+        <v>974259000</v>
       </c>
       <c r="I18" t="n">
-        <v>2349360</v>
+        <v>2794230</v>
       </c>
       <c r="J18" t="n">
         <v>1</v>
       </c>
       <c r="K18" t="n">
-        <v>0</v>
+        <v>11.63</v>
       </c>
       <c r="L18" t="n">
+        <v>31</v>
+      </c>
+      <c r="M18" t="n">
         <v>15</v>
-      </c>
-      <c r="M18" t="n">
-        <v>31</v>
       </c>
       <c r="N18" t="n">
         <v>46</v>
@@ -1322,31 +1322,31 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ITRI11</t>
+          <t>CPTS11</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>77.95</v>
+        <v>7.44</v>
       </c>
       <c r="E19" t="n">
-        <v>13.33</v>
+        <v>6.29</v>
       </c>
       <c r="F19" t="n">
-        <v>13.31</v>
+        <v>12.87</v>
       </c>
       <c r="G19" t="n">
-        <v>0.83</v>
+        <v>0.85</v>
       </c>
       <c r="H19" t="n">
-        <v>487187000</v>
+        <v>2704460000</v>
       </c>
       <c r="I19" t="n">
-        <v>1047070</v>
+        <v>7657600</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1355,13 +1355,13 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="M19" t="n">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="N19" t="n">
-        <v>53</v>
+        <v>48</v>
       </c>
     </row>
     <row r="20">
@@ -1370,31 +1370,31 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>HSAF11</t>
+          <t>CVBI11</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>77.3</v>
+        <v>82.78</v>
       </c>
       <c r="E20" t="n">
-        <v>14.55</v>
+        <v>14.59</v>
       </c>
       <c r="F20" t="n">
-        <v>14.56</v>
+        <v>14.35</v>
       </c>
       <c r="G20" t="n">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
       <c r="H20" t="n">
-        <v>195288000</v>
+        <v>911427000</v>
       </c>
       <c r="I20" t="n">
-        <v>693098</v>
+        <v>3128870</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1403,13 +1403,13 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="M20" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="N20" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="21">
@@ -1418,46 +1418,46 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>RZAK11</t>
+          <t>CPSH11</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Shoppings</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>79.87</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E21" t="n">
-        <v>13.35</v>
+        <v>3.43</v>
       </c>
       <c r="F21" t="n">
-        <v>16.14</v>
+        <v>12.4</v>
       </c>
       <c r="G21" t="n">
-        <v>0.9</v>
+        <v>0.84</v>
       </c>
       <c r="H21" t="n">
-        <v>703486000</v>
+        <v>1194690000</v>
       </c>
       <c r="I21" t="n">
-        <v>1360790</v>
+        <v>5082570</v>
       </c>
       <c r="J21" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>48</v>
+        <v>27</v>
       </c>
       <c r="M21" t="n">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="N21" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="22">
@@ -1466,46 +1466,46 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>KISU11</t>
+          <t>RZTR11</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Terras Agrícolas</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>6.44</v>
+        <v>84.31999999999999</v>
       </c>
       <c r="E22" t="n">
-        <v>13.42</v>
+        <v>9.880000000000001</v>
       </c>
       <c r="F22" t="n">
-        <v>12.83</v>
+        <v>12.65</v>
       </c>
       <c r="G22" t="n">
-        <v>0.8</v>
+        <v>0.86</v>
       </c>
       <c r="H22" t="n">
-        <v>284623000</v>
+        <v>1589580000</v>
       </c>
       <c r="I22" t="n">
-        <v>530294</v>
+        <v>2874000</v>
       </c>
       <c r="J22" t="n">
-        <v>0</v>
+        <v>29</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
       </c>
       <c r="L22" t="n">
-        <v>14</v>
+        <v>31</v>
       </c>
       <c r="M22" t="n">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="N22" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="23">
@@ -1514,46 +1514,46 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CPSH11</t>
+          <t>RBRR11</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Shoppings</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>9.75</v>
+        <v>75.44</v>
       </c>
       <c r="E23" t="n">
-        <v>3.41</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>13.34</v>
+        <v>11.6</v>
       </c>
       <c r="G23" t="n">
-        <v>0.84</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H23" t="n">
-        <v>1200850000</v>
+        <v>1229690000</v>
       </c>
       <c r="I23" t="n">
-        <v>4925140</v>
+        <v>4418800</v>
       </c>
       <c r="J23" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
       </c>
       <c r="L23" t="n">
-        <v>27</v>
+        <v>16</v>
       </c>
       <c r="M23" t="n">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="N23" t="n">
-        <v>59</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24">
@@ -1562,46 +1562,46 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>RBRR11</t>
+          <t>TVRI11</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Escritórios</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>76.59</v>
+        <v>89.36</v>
       </c>
       <c r="E24" t="n">
-        <v>9.06</v>
+        <v>11.76</v>
       </c>
       <c r="F24" t="n">
-        <v>12.7</v>
+        <v>12.63</v>
       </c>
       <c r="G24" t="n">
-        <v>0.82</v>
+        <v>0.86</v>
       </c>
       <c r="H24" t="n">
-        <v>1248440000</v>
+        <v>1422580000</v>
       </c>
       <c r="I24" t="n">
-        <v>4380200</v>
+        <v>877388</v>
       </c>
       <c r="J24" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="K24" t="n">
-        <v>0</v>
+        <v>5.18</v>
       </c>
       <c r="L24" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="M24" t="n">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="N24" t="n">
-        <v>62</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25">
@@ -1610,31 +1610,31 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CVBI11</t>
+          <t>MANA11</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Hedge Fund</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>82.78</v>
+        <v>9.029999999999999</v>
       </c>
       <c r="E25" t="n">
-        <v>14.59</v>
+        <v>10.47</v>
       </c>
       <c r="F25" t="n">
-        <v>14.35</v>
+        <v>26.22</v>
       </c>
       <c r="G25" t="n">
-        <v>0.89</v>
+        <v>0.96</v>
       </c>
       <c r="H25" t="n">
-        <v>911427000</v>
+        <v>338951000</v>
       </c>
       <c r="I25" t="n">
-        <v>3128870</v>
+        <v>1379060</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1643,13 +1643,13 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="M25" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="N25" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="26">
@@ -1658,31 +1658,31 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>VRTA11</t>
+          <t>PORD11</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>73.3</v>
+        <v>8.32</v>
       </c>
       <c r="E26" t="n">
-        <v>13.75</v>
+        <v>13.24</v>
       </c>
       <c r="F26" t="n">
-        <v>13.75</v>
+        <v>12.79</v>
       </c>
       <c r="G26" t="n">
         <v>0.87</v>
       </c>
       <c r="H26" t="n">
-        <v>1142920000</v>
+        <v>310201000</v>
       </c>
       <c r="I26" t="n">
-        <v>2342150</v>
+        <v>624999</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1691,13 +1691,13 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="M26" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="N26" t="n">
-        <v>64</v>
+        <v>59</v>
       </c>
     </row>
     <row r="27">
@@ -1706,31 +1706,31 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>MANA11</t>
+          <t>HFOF11</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>FoF</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>9.130000000000001</v>
+        <v>6.08</v>
       </c>
       <c r="E27" t="n">
-        <v>10.36</v>
+        <v>12.52</v>
       </c>
       <c r="F27" t="n">
-        <v>27.61</v>
+        <v>10.33</v>
       </c>
       <c r="G27" t="n">
-        <v>0.98</v>
+        <v>0.78</v>
       </c>
       <c r="H27" t="n">
-        <v>342705000</v>
+        <v>1335730000</v>
       </c>
       <c r="I27" t="n">
-        <v>1550750</v>
+        <v>2041620</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1739,13 +1739,13 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="M27" t="n">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="N27" t="n">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28">
@@ -1754,31 +1754,31 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PORD11</t>
+          <t>VGIP11</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>8.44</v>
+        <v>75.38</v>
       </c>
       <c r="E28" t="n">
-        <v>13.06</v>
+        <v>12.01</v>
       </c>
       <c r="F28" t="n">
-        <v>13.84</v>
+        <v>11.43</v>
       </c>
       <c r="G28" t="n">
-        <v>0.88</v>
+        <v>0.82</v>
       </c>
       <c r="H28" t="n">
-        <v>314675000</v>
+        <v>888523000</v>
       </c>
       <c r="I28" t="n">
-        <v>521079</v>
+        <v>1956530</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1787,13 +1787,13 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="M28" t="n">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="N28" t="n">
-        <v>66</v>
+        <v>64</v>
       </c>
     </row>
     <row r="29">
@@ -1802,31 +1802,31 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>SNCI11</t>
+          <t>KFOF11</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>FoF</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>85.63</v>
+        <v>75.65000000000001</v>
       </c>
       <c r="E29" t="n">
-        <v>11.29</v>
+        <v>12.41</v>
       </c>
       <c r="F29" t="n">
-        <v>13.68</v>
+        <v>11.4</v>
       </c>
       <c r="G29" t="n">
-        <v>0.88</v>
+        <v>0.82</v>
       </c>
       <c r="H29" t="n">
-        <v>359646000</v>
+        <v>530652000</v>
       </c>
       <c r="I29" t="n">
-        <v>518254</v>
+        <v>1015770</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1835,13 +1835,13 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>41</v>
+        <v>20</v>
       </c>
       <c r="M29" t="n">
-        <v>27</v>
+        <v>45</v>
       </c>
       <c r="N29" t="n">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="30">
@@ -1850,46 +1850,46 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>TVRI11</t>
+          <t>MCLO11</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Escritórios</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>91.41</v>
+        <v>10.88</v>
       </c>
       <c r="E30" t="n">
-        <v>11.5</v>
+        <v>8.6</v>
       </c>
       <c r="F30" t="n">
-        <v>13.62</v>
+        <v>9.65</v>
       </c>
       <c r="G30" t="n">
-        <v>0.88</v>
+        <v>0.79</v>
       </c>
       <c r="H30" t="n">
-        <v>1455220000</v>
+        <v>1356110000</v>
       </c>
       <c r="I30" t="n">
-        <v>1048560</v>
+        <v>2531740</v>
       </c>
       <c r="J30" t="n">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="K30" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>41</v>
+        <v>12</v>
       </c>
       <c r="M30" t="n">
-        <v>28</v>
+        <v>55</v>
       </c>
       <c r="N30" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="31">
@@ -1898,46 +1898,46 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>RZTR11</t>
+          <t>GGRC11</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>86.75</v>
+        <v>9.59</v>
       </c>
       <c r="E31" t="n">
-        <v>9.6</v>
+        <v>5.77</v>
       </c>
       <c r="F31" t="n">
-        <v>13.56</v>
+        <v>12.26</v>
       </c>
       <c r="G31" t="n">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="H31" t="n">
-        <v>1635390000</v>
+        <v>2054650000</v>
       </c>
       <c r="I31" t="n">
-        <v>3044290</v>
+        <v>18370200</v>
       </c>
       <c r="J31" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="M31" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="N31" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="32">
@@ -1946,46 +1946,46 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>VGIR11</t>
+          <t>HSLG11</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>9.6</v>
+        <v>84.15000000000001</v>
       </c>
       <c r="E32" t="n">
-        <v>14.75</v>
+        <v>10.85</v>
       </c>
       <c r="F32" t="n">
-        <v>15.54</v>
+        <v>9.19</v>
       </c>
       <c r="G32" t="n">
-        <v>0.98</v>
+        <v>0.77</v>
       </c>
       <c r="H32" t="n">
-        <v>1402570000</v>
+        <v>1065340000</v>
       </c>
       <c r="I32" t="n">
-        <v>4229740</v>
+        <v>14704900</v>
       </c>
       <c r="J32" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
       </c>
       <c r="L32" t="n">
-        <v>65</v>
+        <v>8</v>
       </c>
       <c r="M32" t="n">
-        <v>7</v>
+        <v>60</v>
       </c>
       <c r="N32" t="n">
-        <v>72</v>
+        <v>68</v>
       </c>
     </row>
     <row r="33">
@@ -1994,46 +1994,46 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MCLO11</t>
+          <t>VGIR11</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>10.4</v>
+        <v>9.56</v>
       </c>
       <c r="E33" t="n">
-        <v>9</v>
+        <v>14.81</v>
       </c>
       <c r="F33" t="n">
-        <v>10.16</v>
+        <v>14.38</v>
       </c>
       <c r="G33" t="n">
-        <v>0.75</v>
+        <v>0.98</v>
       </c>
       <c r="H33" t="n">
-        <v>1296290000</v>
+        <v>1396730000</v>
       </c>
       <c r="I33" t="n">
-        <v>1921040</v>
+        <v>4223880</v>
       </c>
       <c r="J33" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>6</v>
+        <v>60</v>
       </c>
       <c r="M33" t="n">
-        <v>66</v>
+        <v>10</v>
       </c>
       <c r="N33" t="n">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34">
@@ -2042,46 +2042,46 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>HFOF11</t>
+          <t>HGRE11</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Escritórios</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>6.33</v>
+        <v>114.36</v>
       </c>
       <c r="E34" t="n">
-        <v>12.02</v>
+        <v>7.71</v>
       </c>
       <c r="F34" t="n">
-        <v>10.89</v>
+        <v>9.17</v>
       </c>
       <c r="G34" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.78</v>
       </c>
       <c r="H34" t="n">
-        <v>1390660000</v>
+        <v>1351480000</v>
       </c>
       <c r="I34" t="n">
-        <v>2320370</v>
+        <v>2144250</v>
       </c>
       <c r="J34" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="K34" t="n">
-        <v>0</v>
+        <v>5.93</v>
       </c>
       <c r="L34" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M34" t="n">
         <v>61</v>
       </c>
       <c r="N34" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="35">
@@ -2090,31 +2090,31 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>BBFO11</t>
+          <t>BTHF11</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Hedge Fund</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>69.34999999999999</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="E35" t="n">
-        <v>15.5</v>
+        <v>12.06</v>
       </c>
       <c r="F35" t="n">
-        <v>14</v>
+        <v>11.9</v>
       </c>
       <c r="G35" t="n">
-        <v>0.93</v>
+        <v>0.87</v>
       </c>
       <c r="H35" t="n">
-        <v>277670000</v>
+        <v>1790870000</v>
       </c>
       <c r="I35" t="n">
-        <v>508499</v>
+        <v>3084410</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -2123,13 +2123,13 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>55</v>
+        <v>36</v>
       </c>
       <c r="M35" t="n">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="N35" t="n">
-        <v>76</v>
+        <v>71</v>
       </c>
     </row>
     <row r="36">
@@ -2138,46 +2138,46 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>IBBP11</t>
+          <t>RBVA11</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Varejo</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>7.7</v>
+        <v>8.880000000000001</v>
       </c>
       <c r="E36" t="n">
-        <v>6.9</v>
+        <v>7.5</v>
       </c>
       <c r="F36" t="n">
-        <v>11.41</v>
+        <v>10.93</v>
       </c>
       <c r="G36" t="n">
         <v>0.83</v>
       </c>
       <c r="H36" t="n">
-        <v>580354000</v>
+        <v>1386550000</v>
       </c>
       <c r="I36" t="n">
-        <v>551960</v>
+        <v>2113130</v>
       </c>
       <c r="J36" t="n">
-        <v>25</v>
+        <v>74</v>
       </c>
       <c r="K36" t="n">
-        <v>0.22</v>
+        <v>5.97</v>
       </c>
       <c r="L36" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="M36" t="n">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="N36" t="n">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="37">
@@ -2186,46 +2186,46 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>VGIP11</t>
+          <t>VILG11</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>78.37</v>
+        <v>90.23999999999999</v>
       </c>
       <c r="E37" t="n">
-        <v>11.55</v>
+        <v>8.94</v>
       </c>
       <c r="F37" t="n">
-        <v>12.55</v>
+        <v>9.279999999999999</v>
       </c>
       <c r="G37" t="n">
-        <v>0.86</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H37" t="n">
-        <v>923767000</v>
+        <v>1353360000</v>
       </c>
       <c r="I37" t="n">
-        <v>2185120</v>
+        <v>2331440</v>
       </c>
       <c r="J37" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="K37" t="n">
-        <v>0</v>
+        <v>0.51</v>
       </c>
       <c r="L37" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="M37" t="n">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="N37" t="n">
-        <v>78</v>
+        <v>73</v>
       </c>
     </row>
     <row r="38">
@@ -2234,46 +2234,46 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>RCRB11</t>
+          <t>CLIN11</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Escritórios</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>138.98</v>
+        <v>86.48</v>
       </c>
       <c r="E38" t="n">
-        <v>5.2</v>
+        <v>13.82</v>
       </c>
       <c r="F38" t="n">
-        <v>8.6</v>
+        <v>11.96</v>
       </c>
       <c r="G38" t="n">
-        <v>0.7</v>
+        <v>0.88</v>
       </c>
       <c r="H38" t="n">
-        <v>512933000</v>
+        <v>375908000</v>
       </c>
       <c r="I38" t="n">
-        <v>968023</v>
+        <v>649641</v>
       </c>
       <c r="J38" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="M38" t="n">
-        <v>79</v>
+        <v>34</v>
       </c>
       <c r="N38" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
     </row>
     <row r="39">
@@ -2282,46 +2282,46 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>RBVA11</t>
+          <t>RZLC11</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Varejo</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>9</v>
+        <v>1004.35</v>
       </c>
       <c r="E39" t="n">
-        <v>7.4</v>
+        <v>6.99</v>
       </c>
       <c r="F39" t="n">
-        <v>11.88</v>
+        <v>14.46</v>
       </c>
       <c r="G39" t="n">
-        <v>0.84</v>
+        <v>1.01</v>
       </c>
       <c r="H39" t="n">
-        <v>1405290000</v>
+        <v>162668000</v>
       </c>
       <c r="I39" t="n">
-        <v>2258920</v>
+        <v>940304</v>
       </c>
       <c r="J39" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>5.97</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>27</v>
+        <v>67</v>
       </c>
       <c r="M39" t="n">
-        <v>57</v>
+        <v>8</v>
       </c>
       <c r="N39" t="n">
-        <v>84</v>
+        <v>75</v>
       </c>
     </row>
     <row r="40">
@@ -2330,31 +2330,31 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>KFOF11</t>
+          <t>XPCI11</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>78.29000000000001</v>
+        <v>78.75</v>
       </c>
       <c r="E40" t="n">
-        <v>11.99</v>
+        <v>16.36</v>
       </c>
       <c r="F40" t="n">
-        <v>12.07</v>
+        <v>12.3</v>
       </c>
       <c r="G40" t="n">
-        <v>0.85</v>
+        <v>0.89</v>
       </c>
       <c r="H40" t="n">
-        <v>549170000</v>
+        <v>685247000</v>
       </c>
       <c r="I40" t="n">
-        <v>1203180</v>
+        <v>1610120</v>
       </c>
       <c r="J40" t="n">
         <v>0</v>
@@ -2363,13 +2363,13 @@
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="M40" t="n">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="N40" t="n">
-        <v>85</v>
+        <v>76</v>
       </c>
     </row>
     <row r="41">
@@ -2378,46 +2378,46 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>AZPL11</t>
+          <t>ICRI11</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>7.39</v>
+        <v>89.95</v>
       </c>
       <c r="E41" t="n">
-        <v>8.82</v>
+        <v>14.18</v>
       </c>
       <c r="F41" t="n">
-        <v>12.25</v>
+        <v>11.78</v>
       </c>
       <c r="G41" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="H41" t="n">
-        <v>309809000</v>
+        <v>346969000</v>
       </c>
       <c r="I41" t="n">
-        <v>527241</v>
+        <v>635554</v>
       </c>
       <c r="J41" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="M41" t="n">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="N41" t="n">
-        <v>85</v>
+        <v>77</v>
       </c>
     </row>
     <row r="42">
@@ -2426,34 +2426,34 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>RZLC11</t>
+          <t>TRXB11</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Renda Urbana</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>1008.55</v>
+        <v>185.92</v>
       </c>
       <c r="E42" t="n">
-        <v>6.96</v>
+        <v>4.58</v>
       </c>
       <c r="F42" t="n">
-        <v>14.59</v>
+        <v>17.93</v>
       </c>
       <c r="G42" t="n">
-        <v>1.01</v>
+        <v>1.88</v>
       </c>
       <c r="H42" t="n">
-        <v>163348000</v>
+        <v>755955000</v>
       </c>
       <c r="I42" t="n">
-        <v>601732</v>
+        <v>658545</v>
       </c>
       <c r="J42" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
@@ -2462,10 +2462,10 @@
         <v>74</v>
       </c>
       <c r="M42" t="n">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="N42" t="n">
-        <v>87</v>
+        <v>77</v>
       </c>
     </row>
     <row r="43">
@@ -2474,46 +2474,46 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CLIN11</t>
+          <t>AZPL11</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>89.05</v>
+        <v>7.38</v>
       </c>
       <c r="E43" t="n">
-        <v>13.42</v>
+        <v>8.83</v>
       </c>
       <c r="F43" t="n">
-        <v>12.95</v>
+        <v>11.09</v>
       </c>
       <c r="G43" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="H43" t="n">
-        <v>387079000</v>
+        <v>309389000</v>
       </c>
       <c r="I43" t="n">
-        <v>2894300</v>
+        <v>889732</v>
       </c>
       <c r="J43" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="M43" t="n">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="N43" t="n">
-        <v>87</v>
+        <v>78</v>
       </c>
     </row>
     <row r="44">
@@ -2522,46 +2522,46 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>TRXB11</t>
+          <t>BTCI11</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>187.01</v>
+        <v>8.99</v>
       </c>
       <c r="E44" t="n">
-        <v>4.55</v>
+        <v>12.85</v>
       </c>
       <c r="F44" t="n">
-        <v>18.74</v>
+        <v>11.47</v>
       </c>
       <c r="G44" t="n">
-        <v>1.89</v>
+        <v>0.88</v>
       </c>
       <c r="H44" t="n">
-        <v>760387000</v>
+        <v>894695000</v>
       </c>
       <c r="I44" t="n">
-        <v>3127990</v>
+        <v>4890560</v>
       </c>
       <c r="J44" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="K44" t="n">
         <v>0</v>
       </c>
       <c r="L44" t="n">
-        <v>84</v>
+        <v>39</v>
       </c>
       <c r="M44" t="n">
-        <v>3</v>
+        <v>43</v>
       </c>
       <c r="N44" t="n">
-        <v>87</v>
+        <v>82</v>
       </c>
     </row>
     <row r="45">
@@ -2570,46 +2570,46 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ICRI11</t>
+          <t>PMLL11</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Shoppings</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>91.90000000000001</v>
+        <v>100.5</v>
       </c>
       <c r="E45" t="n">
-        <v>13.88</v>
+        <v>10.35</v>
       </c>
       <c r="F45" t="n">
-        <v>12.86</v>
+        <v>10.05</v>
       </c>
       <c r="G45" t="n">
-        <v>0.9</v>
+        <v>0.86</v>
       </c>
       <c r="H45" t="n">
-        <v>354491000</v>
+        <v>1405200000</v>
       </c>
       <c r="I45" t="n">
-        <v>752931</v>
+        <v>4621910</v>
       </c>
       <c r="J45" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="K45" t="n">
-        <v>0</v>
+        <v>3.69</v>
       </c>
       <c r="L45" t="n">
-        <v>48</v>
+        <v>31</v>
       </c>
       <c r="M45" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="N45" t="n">
-        <v>88</v>
+        <v>83</v>
       </c>
     </row>
     <row r="46">
@@ -2618,7 +2618,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>BTAL11</t>
+          <t>XPLG11</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2627,37 +2627,37 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>85.56</v>
+        <v>89.91</v>
       </c>
       <c r="E46" t="n">
-        <v>13.29</v>
+        <v>7</v>
       </c>
       <c r="F46" t="n">
-        <v>7.07</v>
+        <v>9.859999999999999</v>
       </c>
       <c r="G46" t="n">
-        <v>0.74</v>
+        <v>0.85</v>
       </c>
       <c r="H46" t="n">
-        <v>511883000</v>
+        <v>4620480000</v>
       </c>
       <c r="I46" t="n">
-        <v>512875</v>
+        <v>8978070</v>
       </c>
       <c r="J46" t="n">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="K46" t="n">
-        <v>0</v>
+        <v>9.34</v>
       </c>
       <c r="L46" t="n">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="M46" t="n">
-        <v>84</v>
+        <v>54</v>
       </c>
       <c r="N46" t="n">
-        <v>89</v>
+        <v>83</v>
       </c>
     </row>
     <row r="47">
@@ -2666,46 +2666,46 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>HGRE11</t>
+          <t>KNHF11</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Escritórios</t>
+          <t>Hedge Fund</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>121.84</v>
+        <v>90.76000000000001</v>
       </c>
       <c r="E47" t="n">
-        <v>7.24</v>
+        <v>14.11</v>
       </c>
       <c r="F47" t="n">
-        <v>9.359999999999999</v>
+        <v>11.86</v>
       </c>
       <c r="G47" t="n">
-        <v>0.83</v>
+        <v>0.9</v>
       </c>
       <c r="H47" t="n">
-        <v>1439880000</v>
+        <v>1784640000</v>
       </c>
       <c r="I47" t="n">
-        <v>2165750</v>
+        <v>3382020</v>
       </c>
       <c r="J47" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="K47" t="n">
-        <v>5.93</v>
+        <v>0.6</v>
       </c>
       <c r="L47" t="n">
-        <v>20</v>
+        <v>48</v>
       </c>
       <c r="M47" t="n">
-        <v>71</v>
+        <v>36</v>
       </c>
       <c r="N47" t="n">
-        <v>91</v>
+        <v>84</v>
       </c>
     </row>
     <row r="48">
@@ -2714,31 +2714,31 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>BTHF11</t>
+          <t>HGCR11</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>8.94</v>
+        <v>89.67</v>
       </c>
       <c r="E48" t="n">
-        <v>11.73</v>
+        <v>12.39</v>
       </c>
       <c r="F48" t="n">
-        <v>12.72</v>
+        <v>11.79</v>
       </c>
       <c r="G48" t="n">
-        <v>0.9</v>
+        <v>0.91</v>
       </c>
       <c r="H48" t="n">
-        <v>1840270000</v>
+        <v>1382540000</v>
       </c>
       <c r="I48" t="n">
-        <v>3042950</v>
+        <v>3138790</v>
       </c>
       <c r="J48" t="n">
         <v>0</v>
@@ -2747,13 +2747,13 @@
         <v>0</v>
       </c>
       <c r="L48" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="M48" t="n">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="N48" t="n">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="49">
@@ -2762,46 +2762,46 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>PMLL11</t>
+          <t>GARE11</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Shoppings</t>
+          <t>Multicategoria</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>100.6</v>
+        <v>8.16</v>
       </c>
       <c r="E49" t="n">
-        <v>10.34</v>
+        <v>5.25</v>
       </c>
       <c r="F49" t="n">
-        <v>10.99</v>
+        <v>10.96</v>
       </c>
       <c r="G49" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="H49" t="n">
-        <v>1406600000</v>
+        <v>2359760000</v>
       </c>
       <c r="I49" t="n">
-        <v>4738330</v>
+        <v>10103400</v>
       </c>
       <c r="J49" t="n">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="K49" t="n">
-        <v>3.69</v>
+        <v>0</v>
       </c>
       <c r="L49" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="M49" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
       <c r="N49" t="n">
-        <v>93</v>
+        <v>87</v>
       </c>
     </row>
     <row r="50">
@@ -2810,46 +2810,46 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>GARE11</t>
+          <t>FATN11</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Escritórios</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>8.17</v>
+        <v>77.90000000000001</v>
       </c>
       <c r="E50" t="n">
-        <v>5.24</v>
+        <v>5.38</v>
       </c>
       <c r="F50" t="n">
-        <v>12.07</v>
+        <v>7.98</v>
       </c>
       <c r="G50" t="n">
-        <v>0.88</v>
+        <v>0.8</v>
       </c>
       <c r="H50" t="n">
-        <v>2362650000</v>
+        <v>526469000</v>
       </c>
       <c r="I50" t="n">
-        <v>11072400</v>
+        <v>2327470</v>
       </c>
       <c r="J50" t="n">
-        <v>3</v>
+        <v>60</v>
       </c>
       <c r="K50" t="n">
-        <v>0</v>
+        <v>20.92</v>
       </c>
       <c r="L50" t="n">
-        <v>41</v>
+        <v>15</v>
       </c>
       <c r="M50" t="n">
-        <v>53</v>
+        <v>73</v>
       </c>
       <c r="N50" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
     </row>
     <row r="51">
@@ -2858,46 +2858,46 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>BTCI11</t>
+          <t>MALL11</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Shoppings</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>9.140000000000001</v>
+        <v>100.03</v>
       </c>
       <c r="E51" t="n">
-        <v>12.64</v>
+        <v>14.22</v>
       </c>
       <c r="F51" t="n">
-        <v>12.48</v>
+        <v>8.91</v>
       </c>
       <c r="G51" t="n">
-        <v>0.89</v>
+        <v>0.83</v>
       </c>
       <c r="H51" t="n">
-        <v>909623000</v>
+        <v>1398630000</v>
       </c>
       <c r="I51" t="n">
-        <v>5600480</v>
+        <v>1520130</v>
       </c>
       <c r="J51" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K51" t="n">
-        <v>0</v>
+        <v>3.64</v>
       </c>
       <c r="L51" t="n">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="M51" t="n">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="N51" t="n">
-        <v>94</v>
+        <v>88</v>
       </c>
     </row>
     <row r="52">
@@ -2906,7 +2906,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>XPCI11</t>
+          <t>SNEL11</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2915,37 +2915,37 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>82.88</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="E52" t="n">
-        <v>15.55</v>
+        <v>5.74</v>
       </c>
       <c r="F52" t="n">
-        <v>12.96</v>
+        <v>12.85</v>
       </c>
       <c r="G52" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.05</v>
       </c>
       <c r="H52" t="n">
-        <v>721185000</v>
+        <v>925118000</v>
       </c>
       <c r="I52" t="n">
-        <v>1929520</v>
+        <v>6874160</v>
       </c>
       <c r="J52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K52" t="n">
         <v>0</v>
       </c>
       <c r="L52" t="n">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="M52" t="n">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="N52" t="n">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="53">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>VILG11</t>
+          <t>LVBI11</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2963,37 +2963,37 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>94</v>
+        <v>99.34999999999999</v>
       </c>
       <c r="E53" t="n">
-        <v>8.58</v>
+        <v>9.02</v>
       </c>
       <c r="F53" t="n">
-        <v>9.75</v>
+        <v>8.18</v>
       </c>
       <c r="G53" t="n">
-        <v>0.84</v>
+        <v>0.82</v>
       </c>
       <c r="H53" t="n">
-        <v>1409760000</v>
+        <v>1601380000</v>
       </c>
       <c r="I53" t="n">
-        <v>2937140</v>
+        <v>3192610</v>
       </c>
       <c r="J53" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="K53" t="n">
-        <v>0.51</v>
+        <v>5.75</v>
       </c>
       <c r="L53" t="n">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="M53" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="N53" t="n">
-        <v>96</v>
+        <v>91</v>
       </c>
     </row>
     <row r="54">
@@ -3002,46 +3002,46 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TRXF11</t>
+          <t>MXRF11</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>91.34999999999999</v>
+        <v>9.35</v>
       </c>
       <c r="E54" t="n">
-        <v>4.65</v>
+        <v>11.23</v>
       </c>
       <c r="F54" t="n">
-        <v>12.77</v>
+        <v>12.52</v>
       </c>
       <c r="G54" t="n">
-        <v>0.93</v>
+        <v>1</v>
       </c>
       <c r="H54" t="n">
-        <v>5703040000</v>
+        <v>4303520000</v>
       </c>
       <c r="I54" t="n">
-        <v>21248200</v>
+        <v>15001600</v>
       </c>
       <c r="J54" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="K54" t="n">
         <v>0</v>
       </c>
       <c r="L54" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="M54" t="n">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="N54" t="n">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="55">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>KNUQ11</t>
+          <t>RINV11</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -3059,22 +3059,22 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>105.32</v>
+        <v>101.25</v>
       </c>
       <c r="E55" t="n">
-        <v>12.19</v>
+        <v>8.779999999999999</v>
       </c>
       <c r="F55" t="n">
-        <v>14.03</v>
+        <v>11.62</v>
       </c>
       <c r="G55" t="n">
-        <v>1.04</v>
+        <v>0.95</v>
       </c>
       <c r="H55" t="n">
-        <v>2262770000</v>
+        <v>509457000</v>
       </c>
       <c r="I55" t="n">
-        <v>4784120</v>
+        <v>549888</v>
       </c>
       <c r="J55" t="n">
         <v>0</v>
@@ -3083,13 +3083,13 @@
         <v>0</v>
       </c>
       <c r="L55" t="n">
-        <v>77</v>
+        <v>55</v>
       </c>
       <c r="M55" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="N55" t="n">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="56">
@@ -3098,46 +3098,46 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>MALL11</t>
+          <t>KNUQ11</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Shoppings</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>100.03</v>
+        <v>104.14</v>
       </c>
       <c r="E56" t="n">
-        <v>14.22</v>
+        <v>12.33</v>
       </c>
       <c r="F56" t="n">
-        <v>8.91</v>
+        <v>12.62</v>
       </c>
       <c r="G56" t="n">
-        <v>0.83</v>
+        <v>1.03</v>
       </c>
       <c r="H56" t="n">
-        <v>1398630000</v>
+        <v>2237420000</v>
       </c>
       <c r="I56" t="n">
-        <v>1520130</v>
+        <v>4129240</v>
       </c>
       <c r="J56" t="n">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="K56" t="n">
-        <v>3.64</v>
+        <v>0</v>
       </c>
       <c r="L56" t="n">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="M56" t="n">
-        <v>77</v>
+        <v>27</v>
       </c>
       <c r="N56" t="n">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="57">
@@ -3146,46 +3146,46 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>XPLG11</t>
+          <t>MCCI11</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="E57" t="n">
-        <v>6.92</v>
+        <v>11.53</v>
       </c>
       <c r="F57" t="n">
-        <v>10.72</v>
+        <v>11.57</v>
       </c>
       <c r="G57" t="n">
-        <v>0.86</v>
+        <v>0.98</v>
       </c>
       <c r="H57" t="n">
-        <v>4676500000</v>
+        <v>1577280000</v>
       </c>
       <c r="I57" t="n">
-        <v>9718040</v>
+        <v>5012850</v>
       </c>
       <c r="J57" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="K57" t="n">
-        <v>9.34</v>
+        <v>0</v>
       </c>
       <c r="L57" t="n">
-        <v>33</v>
+        <v>60</v>
       </c>
       <c r="M57" t="n">
-        <v>64</v>
+        <v>41</v>
       </c>
       <c r="N57" t="n">
-        <v>97</v>
+        <v>101</v>
       </c>
     </row>
     <row r="58">
@@ -3194,43 +3194,43 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>FATN11</t>
+          <t>KNCR11</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>80.13</v>
+        <v>105.6</v>
       </c>
       <c r="E58" t="n">
-        <v>5.23</v>
+        <v>9.93</v>
       </c>
       <c r="F58" t="n">
-        <v>7.83</v>
+        <v>12.1</v>
       </c>
       <c r="G58" t="n">
-        <v>0.83</v>
+        <v>1.03</v>
       </c>
       <c r="H58" t="n">
-        <v>541539000</v>
+        <v>11308700000</v>
       </c>
       <c r="I58" t="n">
-        <v>2405970</v>
+        <v>20928500</v>
       </c>
       <c r="J58" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="K58" t="n">
-        <v>20.92</v>
+        <v>0</v>
       </c>
       <c r="L58" t="n">
-        <v>20</v>
+        <v>69</v>
       </c>
       <c r="M58" t="n">
-        <v>82</v>
+        <v>33</v>
       </c>
       <c r="N58" t="n">
         <v>102</v>
@@ -3242,46 +3242,46 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>HSLG11</t>
+          <t>AFHI11</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>91.83</v>
+        <v>94</v>
       </c>
       <c r="E59" t="n">
-        <v>9.94</v>
+        <v>11.59</v>
       </c>
       <c r="F59" t="n">
-        <v>9.199999999999999</v>
+        <v>11.48</v>
       </c>
       <c r="G59" t="n">
-        <v>0.84</v>
+        <v>0.99</v>
       </c>
       <c r="H59" t="n">
-        <v>1162570000</v>
+        <v>450184000</v>
       </c>
       <c r="I59" t="n">
-        <v>1090730</v>
+        <v>713635</v>
       </c>
       <c r="J59" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="K59" t="n">
         <v>0</v>
       </c>
       <c r="L59" t="n">
-        <v>27</v>
+        <v>63</v>
       </c>
       <c r="M59" t="n">
-        <v>75</v>
+        <v>42</v>
       </c>
       <c r="N59" t="n">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="60">
@@ -3290,46 +3290,46 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>SNEL11</t>
+          <t>KNIP11</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Multicategoria</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>8.4</v>
+        <v>89.40000000000001</v>
       </c>
       <c r="E60" t="n">
-        <v>5.71</v>
+        <v>12.94</v>
       </c>
       <c r="F60" t="n">
-        <v>13.95</v>
+        <v>10.09</v>
       </c>
       <c r="G60" t="n">
-        <v>1.05</v>
+        <v>0.96</v>
       </c>
       <c r="H60" t="n">
-        <v>929545000</v>
+        <v>7158990000</v>
       </c>
       <c r="I60" t="n">
-        <v>6844870</v>
+        <v>10781300</v>
       </c>
       <c r="J60" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K60" t="n">
         <v>0</v>
       </c>
       <c r="L60" t="n">
-        <v>80</v>
+        <v>56</v>
       </c>
       <c r="M60" t="n">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="N60" t="n">
-        <v>102</v>
+        <v>107</v>
       </c>
     </row>
     <row r="61">
@@ -3338,46 +3338,46 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>GGRC11</t>
+          <t>HGRU11</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Renda Urbana</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>9.92</v>
+        <v>116.8</v>
       </c>
       <c r="E61" t="n">
-        <v>5.58</v>
+        <v>8.52</v>
       </c>
       <c r="F61" t="n">
-        <v>11.97</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="G61" t="n">
-        <v>0.9</v>
+        <v>0.91</v>
       </c>
       <c r="H61" t="n">
-        <v>2125360000</v>
+        <v>2714200000</v>
       </c>
       <c r="I61" t="n">
-        <v>15041400</v>
+        <v>6286520</v>
       </c>
       <c r="J61" t="n">
-        <v>42</v>
+        <v>100</v>
       </c>
       <c r="K61" t="n">
-        <v>0</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="L61" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="M61" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="N61" t="n">
-        <v>104</v>
+        <v>107</v>
       </c>
     </row>
     <row r="62">
@@ -3386,46 +3386,46 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>HGCR11</t>
+          <t>HGLG11</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Multicategoria</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>93.40000000000001</v>
+        <v>145.55</v>
       </c>
       <c r="E62" t="n">
-        <v>11.89</v>
+        <v>6.68</v>
       </c>
       <c r="F62" t="n">
-        <v>12.55</v>
+        <v>8.19</v>
       </c>
       <c r="G62" t="n">
-        <v>0.95</v>
+        <v>0.88</v>
       </c>
       <c r="H62" t="n">
-        <v>1440050000</v>
+        <v>6637330000</v>
       </c>
       <c r="I62" t="n">
-        <v>3162580</v>
+        <v>17266200</v>
       </c>
       <c r="J62" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="K62" t="n">
-        <v>0</v>
+        <v>3.23</v>
       </c>
       <c r="L62" t="n">
-        <v>62</v>
+        <v>39</v>
       </c>
       <c r="M62" t="n">
-        <v>45</v>
+        <v>70</v>
       </c>
       <c r="N62" t="n">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="63">
@@ -3434,46 +3434,46 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>KNHF11</t>
+          <t>HGBS11</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Shoppings</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>95.5</v>
+        <v>18.81</v>
       </c>
       <c r="E63" t="n">
-        <v>13.41</v>
+        <v>8.130000000000001</v>
       </c>
       <c r="F63" t="n">
-        <v>12.43</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G63" t="n">
-        <v>0.95</v>
+        <v>0.92</v>
       </c>
       <c r="H63" t="n">
-        <v>1877840000</v>
+        <v>2715330000</v>
       </c>
       <c r="I63" t="n">
-        <v>3555840</v>
+        <v>4397500</v>
       </c>
       <c r="J63" t="n">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="K63" t="n">
-        <v>0.6</v>
+        <v>4.31</v>
       </c>
       <c r="L63" t="n">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="M63" t="n">
-        <v>49</v>
+        <v>59</v>
       </c>
       <c r="N63" t="n">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="64">
@@ -3482,46 +3482,46 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MXRF11</t>
+          <t>VISC11</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Shoppings</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>9.67</v>
+        <v>103.24</v>
       </c>
       <c r="E64" t="n">
-        <v>10.85</v>
+        <v>5.88</v>
       </c>
       <c r="F64" t="n">
-        <v>13.26</v>
+        <v>8.66</v>
       </c>
       <c r="G64" t="n">
-        <v>1.03</v>
+        <v>0.89</v>
       </c>
       <c r="H64" t="n">
-        <v>4450810000</v>
+        <v>2976270000</v>
       </c>
       <c r="I64" t="n">
-        <v>14687200</v>
+        <v>4675760</v>
       </c>
       <c r="J64" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="K64" t="n">
-        <v>0</v>
+        <v>5.74</v>
       </c>
       <c r="L64" t="n">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="M64" t="n">
-        <v>35</v>
+        <v>67</v>
       </c>
       <c r="N64" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="65">
@@ -3530,43 +3530,43 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>LVBI11</t>
+          <t>ALZR11</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Multicategoria</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>103.96</v>
+        <v>9.869999999999999</v>
       </c>
       <c r="E65" t="n">
-        <v>8.619999999999999</v>
+        <v>7.69</v>
       </c>
       <c r="F65" t="n">
-        <v>8.59</v>
+        <v>9.16</v>
       </c>
       <c r="G65" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="H65" t="n">
-        <v>1675690000</v>
+        <v>1623740000</v>
       </c>
       <c r="I65" t="n">
-        <v>3189810</v>
+        <v>3107340</v>
       </c>
       <c r="J65" t="n">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="K65" t="n">
-        <v>5.75</v>
+        <v>12.46</v>
       </c>
       <c r="L65" t="n">
-        <v>33</v>
+        <v>51</v>
       </c>
       <c r="M65" t="n">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="N65" t="n">
         <v>113</v>
@@ -3578,46 +3578,46 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>HTMX11</t>
+          <t>KNSC11</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Hotel</t>
+          <t>Multicategoria</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>140.96</v>
+        <v>8.960000000000001</v>
       </c>
       <c r="E66" t="n">
-        <v>7.43</v>
+        <v>13.76</v>
       </c>
       <c r="F66" t="n">
-        <v>12.05</v>
+        <v>11.31</v>
       </c>
       <c r="G66" t="n">
-        <v>0.9399999999999999</v>
+        <v>1.02</v>
       </c>
       <c r="H66" t="n">
-        <v>407106000</v>
+        <v>1811730000</v>
       </c>
       <c r="I66" t="n">
-        <v>512192</v>
+        <v>4200810</v>
       </c>
       <c r="J66" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K66" t="n">
         <v>0</v>
       </c>
       <c r="L66" t="n">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="M66" t="n">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="N66" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="67">
@@ -3626,46 +3626,46 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>CPLG11</t>
+          <t>HSRE11</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Renda Urbana</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>10.94</v>
+        <v>86.45</v>
       </c>
       <c r="E67" t="n">
-        <v>0.89</v>
+        <v>7.39</v>
       </c>
       <c r="F67" t="n">
-        <v>13.05</v>
+        <v>10.04</v>
       </c>
       <c r="G67" t="n">
-        <v>1.04</v>
+        <v>1</v>
       </c>
       <c r="H67" t="n">
-        <v>616532000</v>
+        <v>769295000</v>
       </c>
       <c r="I67" t="n">
-        <v>834067</v>
+        <v>3770130</v>
       </c>
       <c r="J67" t="n">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
       </c>
       <c r="L67" t="n">
-        <v>77</v>
+        <v>65</v>
       </c>
       <c r="M67" t="n">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="N67" t="n">
-        <v>114</v>
+        <v>118</v>
       </c>
     </row>
     <row r="68">
@@ -3674,7 +3674,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>KNCR11</t>
+          <t>KNHY11</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -3683,22 +3683,22 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>107.58</v>
+        <v>97.68000000000001</v>
       </c>
       <c r="E68" t="n">
-        <v>9.75</v>
+        <v>12.27</v>
       </c>
       <c r="F68" t="n">
-        <v>13.25</v>
+        <v>9.58</v>
       </c>
       <c r="G68" t="n">
-        <v>1.05</v>
+        <v>0.99</v>
       </c>
       <c r="H68" t="n">
-        <v>11520700000</v>
+        <v>3044990000</v>
       </c>
       <c r="I68" t="n">
-        <v>21806100</v>
+        <v>3842470</v>
       </c>
       <c r="J68" t="n">
         <v>0</v>
@@ -3707,13 +3707,13 @@
         <v>0</v>
       </c>
       <c r="L68" t="n">
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="M68" t="n">
-        <v>36</v>
+        <v>56</v>
       </c>
       <c r="N68" t="n">
-        <v>116</v>
+        <v>119</v>
       </c>
     </row>
     <row r="69">
@@ -3722,46 +3722,46 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>AFHI11</t>
+          <t>HPDP11</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Shoppings</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>94.7</v>
+        <v>87.98999999999999</v>
       </c>
       <c r="E69" t="n">
-        <v>11.5</v>
+        <v>4.34</v>
       </c>
       <c r="F69" t="n">
-        <v>12.51</v>
+        <v>8.109999999999999</v>
       </c>
       <c r="G69" t="n">
-        <v>0.99</v>
+        <v>0.92</v>
       </c>
       <c r="H69" t="n">
-        <v>453536000</v>
+        <v>620417000</v>
       </c>
       <c r="I69" t="n">
-        <v>717838</v>
+        <v>828346</v>
       </c>
       <c r="J69" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K69" t="n">
-        <v>0</v>
+        <v>1.65</v>
       </c>
       <c r="L69" t="n">
-        <v>69</v>
+        <v>51</v>
       </c>
       <c r="M69" t="n">
-        <v>47</v>
+        <v>72</v>
       </c>
       <c r="N69" t="n">
-        <v>116</v>
+        <v>123</v>
       </c>
     </row>
     <row r="70">
@@ -3770,46 +3770,46 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MCCI11</t>
+          <t>BRCO11</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>94.40000000000001</v>
+        <v>111.9</v>
       </c>
       <c r="E70" t="n">
-        <v>11.36</v>
+        <v>7.28</v>
       </c>
       <c r="F70" t="n">
-        <v>12.33</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="G70" t="n">
-        <v>1</v>
+        <v>0.97</v>
       </c>
       <c r="H70" t="n">
-        <v>1601030000</v>
+        <v>2016580000</v>
       </c>
       <c r="I70" t="n">
-        <v>5426680</v>
+        <v>4908510</v>
       </c>
       <c r="J70" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="K70" t="n">
-        <v>0</v>
+        <v>12.62</v>
       </c>
       <c r="L70" t="n">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="M70" t="n">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="N70" t="n">
-        <v>121</v>
+        <v>124</v>
       </c>
     </row>
     <row r="71">
@@ -3818,46 +3818,46 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>ALZR11</t>
+          <t>PQDP11</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Shoppings</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>9.91</v>
+        <v>2514.96</v>
       </c>
       <c r="E71" t="n">
-        <v>7.65</v>
+        <v>5.19</v>
       </c>
       <c r="F71" t="n">
-        <v>10.05</v>
+        <v>8.25</v>
       </c>
       <c r="G71" t="n">
-        <v>0.93</v>
+        <v>0.97</v>
       </c>
       <c r="H71" t="n">
-        <v>1630320000</v>
+        <v>614186000</v>
       </c>
       <c r="I71" t="n">
-        <v>3394880</v>
+        <v>2085960</v>
       </c>
       <c r="J71" t="n">
-        <v>22</v>
+        <v>1</v>
       </c>
       <c r="K71" t="n">
-        <v>12.46</v>
+        <v>0.66</v>
       </c>
       <c r="L71" t="n">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="M71" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="N71" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="72">
@@ -3866,46 +3866,46 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>HGBS11</t>
+          <t>KNRI11</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Shoppings</t>
+          <t>Multicategoria</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>19.25</v>
+        <v>152.18</v>
       </c>
       <c r="E72" t="n">
-        <v>7.94</v>
+        <v>7.58</v>
       </c>
       <c r="F72" t="n">
-        <v>9.84</v>
+        <v>7.71</v>
       </c>
       <c r="G72" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="H72" t="n">
-        <v>2778850000</v>
+        <v>4292090000</v>
       </c>
       <c r="I72" t="n">
-        <v>5153880</v>
+        <v>7483780</v>
       </c>
       <c r="J72" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K72" t="n">
-        <v>4.31</v>
+        <v>0.09</v>
       </c>
       <c r="L72" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="M72" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="N72" t="n">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="73">
@@ -3914,7 +3914,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>HGLG11</t>
+          <t>BTLG11</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -3923,37 +3923,37 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>149.01</v>
+        <v>100.38</v>
       </c>
       <c r="E73" t="n">
-        <v>6.53</v>
+        <v>6</v>
       </c>
       <c r="F73" t="n">
-        <v>8.800000000000001</v>
+        <v>8.57</v>
       </c>
       <c r="G73" t="n">
-        <v>0.9</v>
+        <v>0.98</v>
       </c>
       <c r="H73" t="n">
-        <v>6795120000</v>
+        <v>6965330000</v>
       </c>
       <c r="I73" t="n">
-        <v>15162800</v>
+        <v>11570200</v>
       </c>
       <c r="J73" t="n">
+        <v>31</v>
+      </c>
+      <c r="K73" t="n">
+        <v>5.06</v>
+      </c>
+      <c r="L73" t="n">
         <v>60</v>
       </c>
-      <c r="K73" t="n">
-        <v>3.23</v>
-      </c>
-      <c r="L73" t="n">
-        <v>48</v>
-      </c>
       <c r="M73" t="n">
-        <v>78</v>
+        <v>68</v>
       </c>
       <c r="N73" t="n">
-        <v>126</v>
+        <v>128</v>
       </c>
     </row>
     <row r="74">
@@ -3962,46 +3962,46 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>VISC11</t>
+          <t>CPUR11</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Shoppings</t>
+          <t>Multicategoria</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>105.1</v>
+        <v>10.97</v>
       </c>
       <c r="E74" t="n">
-        <v>5.77</v>
+        <v>6.87</v>
       </c>
       <c r="F74" t="n">
-        <v>9.34</v>
+        <v>9.050000000000001</v>
       </c>
       <c r="G74" t="n">
-        <v>0.91</v>
+        <v>1.13</v>
       </c>
       <c r="H74" t="n">
-        <v>3029890000</v>
+        <v>744048000</v>
       </c>
       <c r="I74" t="n">
-        <v>7087390</v>
+        <v>13844800</v>
       </c>
       <c r="J74" t="n">
-        <v>32</v>
+        <v>18</v>
       </c>
       <c r="K74" t="n">
-        <v>5.74</v>
+        <v>0.62</v>
       </c>
       <c r="L74" t="n">
-        <v>54</v>
+        <v>72</v>
       </c>
       <c r="M74" t="n">
-        <v>73</v>
+        <v>63</v>
       </c>
       <c r="N74" t="n">
-        <v>127</v>
+        <v>135</v>
       </c>
     </row>
     <row r="75">
@@ -4010,7 +4010,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>KNSC11</t>
+          <t>HBCR11</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -4019,517 +4019,37 @@
         </is>
       </c>
       <c r="D75" t="n">
-        <v>9.15</v>
+        <v>153.52</v>
       </c>
       <c r="E75" t="n">
-        <v>13.47</v>
+        <v>5.13</v>
       </c>
       <c r="F75" t="n">
-        <v>12.32</v>
+        <v>8.94</v>
       </c>
       <c r="G75" t="n">
-        <v>1.04</v>
+        <v>1.31</v>
       </c>
       <c r="H75" t="n">
-        <v>1850150000</v>
+        <v>245632000</v>
       </c>
       <c r="I75" t="n">
-        <v>4596550</v>
+        <v>8768020</v>
       </c>
       <c r="J75" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K75" t="n">
         <v>0</v>
       </c>
       <c r="L75" t="n">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="M75" t="n">
-        <v>51</v>
+        <v>64</v>
       </c>
       <c r="N75" t="n">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="n">
-        <v>75</v>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>HSRE11</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>Outros</t>
-        </is>
-      </c>
-      <c r="D76" t="n">
-        <v>86.23</v>
-      </c>
-      <c r="E76" t="n">
-        <v>7.41</v>
-      </c>
-      <c r="F76" t="n">
-        <v>11.03</v>
-      </c>
-      <c r="G76" t="n">
-        <v>1</v>
-      </c>
-      <c r="H76" t="n">
-        <v>767337000</v>
-      </c>
-      <c r="I76" t="n">
-        <v>5378940</v>
-      </c>
-      <c r="J76" t="n">
-        <v>22</v>
-      </c>
-      <c r="K76" t="n">
-        <v>0</v>
-      </c>
-      <c r="L76" t="n">
-        <v>71</v>
-      </c>
-      <c r="M76" t="n">
-        <v>59</v>
-      </c>
-      <c r="N76" t="n">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="n">
-        <v>76</v>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>KNIP11</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>Multicategoria</t>
-        </is>
-      </c>
-      <c r="D77" t="n">
-        <v>92.04000000000001</v>
-      </c>
-      <c r="E77" t="n">
-        <v>12.56</v>
-      </c>
-      <c r="F77" t="n">
-        <v>10.76</v>
-      </c>
-      <c r="G77" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="H77" t="n">
-        <v>7370400000</v>
-      </c>
-      <c r="I77" t="n">
-        <v>11338600</v>
-      </c>
-      <c r="J77" t="n">
-        <v>0</v>
-      </c>
-      <c r="K77" t="n">
-        <v>0</v>
-      </c>
-      <c r="L77" t="n">
-        <v>69</v>
-      </c>
-      <c r="M77" t="n">
-        <v>62</v>
-      </c>
-      <c r="N77" t="n">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="n">
-        <v>77</v>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>PQDP11</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>Shoppings</t>
-        </is>
-      </c>
-      <c r="D78" t="n">
-        <v>2452</v>
-      </c>
-      <c r="E78" t="n">
-        <v>5.33</v>
-      </c>
-      <c r="F78" t="n">
-        <v>9.26</v>
-      </c>
-      <c r="G78" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="H78" t="n">
-        <v>598810000</v>
-      </c>
-      <c r="I78" t="n">
-        <v>1434810</v>
-      </c>
-      <c r="J78" t="n">
-        <v>1</v>
-      </c>
-      <c r="K78" t="n">
-        <v>0.66</v>
-      </c>
-      <c r="L78" t="n">
-        <v>58</v>
-      </c>
-      <c r="M78" t="n">
-        <v>74</v>
-      </c>
-      <c r="N78" t="n">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="n">
-        <v>78</v>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>BRCO11</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>Logística</t>
-        </is>
-      </c>
-      <c r="D79" t="n">
-        <v>113.6</v>
-      </c>
-      <c r="E79" t="n">
-        <v>7.17</v>
-      </c>
-      <c r="F79" t="n">
-        <v>9.5</v>
-      </c>
-      <c r="G79" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="H79" t="n">
-        <v>2047220000</v>
-      </c>
-      <c r="I79" t="n">
-        <v>5646640</v>
-      </c>
-      <c r="J79" t="n">
-        <v>14</v>
-      </c>
-      <c r="K79" t="n">
-        <v>12.62</v>
-      </c>
-      <c r="L79" t="n">
-        <v>65</v>
-      </c>
-      <c r="M79" t="n">
-        <v>70</v>
-      </c>
-      <c r="N79" t="n">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="n">
-        <v>79</v>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>HGRU11</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>Outros</t>
-        </is>
-      </c>
-      <c r="D80" t="n">
-        <v>126</v>
-      </c>
-      <c r="E80" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="F80" t="n">
-        <v>9.359999999999999</v>
-      </c>
-      <c r="G80" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="H80" t="n">
-        <v>2927990000</v>
-      </c>
-      <c r="I80" t="n">
-        <v>5717620</v>
-      </c>
-      <c r="J80" t="n">
-        <v>100</v>
-      </c>
-      <c r="K80" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="L80" t="n">
-        <v>65</v>
-      </c>
-      <c r="M80" t="n">
-        <v>71</v>
-      </c>
-      <c r="N80" t="n">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="n">
-        <v>80</v>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>KNHY11</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>Multicategoria</t>
-        </is>
-      </c>
-      <c r="D81" t="n">
-        <v>99.84999999999999</v>
-      </c>
-      <c r="E81" t="n">
-        <v>12</v>
-      </c>
-      <c r="F81" t="n">
-        <v>10.74</v>
-      </c>
-      <c r="G81" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="H81" t="n">
-        <v>3112630000</v>
-      </c>
-      <c r="I81" t="n">
-        <v>3231860</v>
-      </c>
-      <c r="J81" t="n">
-        <v>0</v>
-      </c>
-      <c r="K81" t="n">
-        <v>0</v>
-      </c>
-      <c r="L81" t="n">
-        <v>74</v>
-      </c>
-      <c r="M81" t="n">
-        <v>63</v>
-      </c>
-      <c r="N81" t="n">
         <v>137</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="n">
-        <v>81</v>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>KNRI11</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>Multicategoria</t>
-        </is>
-      </c>
-      <c r="D82" t="n">
-        <v>156.29</v>
-      </c>
-      <c r="E82" t="n">
-        <v>7.38</v>
-      </c>
-      <c r="F82" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="G82" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="H82" t="n">
-        <v>4408010000</v>
-      </c>
-      <c r="I82" t="n">
-        <v>8123860</v>
-      </c>
-      <c r="J82" t="n">
-        <v>18</v>
-      </c>
-      <c r="K82" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="L82" t="n">
-        <v>64</v>
-      </c>
-      <c r="M82" t="n">
-        <v>81</v>
-      </c>
-      <c r="N82" t="n">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="n">
-        <v>82</v>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>BTLG11</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>Multicategoria</t>
-        </is>
-      </c>
-      <c r="D83" t="n">
-        <v>102.39</v>
-      </c>
-      <c r="E83" t="n">
-        <v>5.88</v>
-      </c>
-      <c r="F83" t="n">
-        <v>9.15</v>
-      </c>
-      <c r="G83" t="n">
-        <v>1</v>
-      </c>
-      <c r="H83" t="n">
-        <v>7104810000</v>
-      </c>
-      <c r="I83" t="n">
-        <v>11878100</v>
-      </c>
-      <c r="J83" t="n">
-        <v>31</v>
-      </c>
-      <c r="K83" t="n">
-        <v>5.06</v>
-      </c>
-      <c r="L83" t="n">
-        <v>71</v>
-      </c>
-      <c r="M83" t="n">
-        <v>76</v>
-      </c>
-      <c r="N83" t="n">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="n">
-        <v>83</v>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>CPUR11</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>Multicategoria</t>
-        </is>
-      </c>
-      <c r="D84" t="n">
-        <v>10.31</v>
-      </c>
-      <c r="E84" t="n">
-        <v>7.31</v>
-      </c>
-      <c r="F84" t="n">
-        <v>10.21</v>
-      </c>
-      <c r="G84" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="H84" t="n">
-        <v>699283000</v>
-      </c>
-      <c r="I84" t="n">
-        <v>1499900</v>
-      </c>
-      <c r="J84" t="n">
-        <v>18</v>
-      </c>
-      <c r="K84" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="L84" t="n">
-        <v>82</v>
-      </c>
-      <c r="M84" t="n">
-        <v>65</v>
-      </c>
-      <c r="N84" t="n">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="n">
-        <v>84</v>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>SHPP11</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>Multicategoria</t>
-        </is>
-      </c>
-      <c r="D85" t="n">
-        <v>10.88</v>
-      </c>
-      <c r="E85" t="n">
-        <v>8.08</v>
-      </c>
-      <c r="F85" t="n">
-        <v>7.39</v>
-      </c>
-      <c r="G85" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="H85" t="n">
-        <v>555614000</v>
-      </c>
-      <c r="I85" t="n">
-        <v>3202740</v>
-      </c>
-      <c r="J85" t="n">
-        <v>0</v>
-      </c>
-      <c r="K85" t="n">
-        <v>0</v>
-      </c>
-      <c r="L85" t="n">
-        <v>82</v>
-      </c>
-      <c r="M85" t="n">
-        <v>83</v>
-      </c>
-      <c r="N85" t="n">
-        <v>165</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: implementação da aba de análise de Fundos Imobiliários por IA
</commit_message>
<xml_diff>
--- a/ranking_fiis.xlsx
+++ b/ranking_fiis.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N75"/>
+  <dimension ref="A1:N85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -506,31 +506,31 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LIFE11</t>
+          <t>OUJP11</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Residencial</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>7.02</v>
+        <v>70.16</v>
       </c>
       <c r="E2" t="n">
-        <v>15.78</v>
+        <v>20.66</v>
       </c>
       <c r="F2" t="n">
-        <v>18.22</v>
+        <v>19.87</v>
       </c>
       <c r="G2" t="n">
-        <v>0.73</v>
+        <v>0.7</v>
       </c>
       <c r="H2" t="n">
-        <v>279126000</v>
+        <v>228187000</v>
       </c>
       <c r="I2" t="n">
-        <v>803094</v>
+        <v>573530</v>
       </c>
       <c r="J2" t="n">
         <v>0</v>
@@ -539,13 +539,13 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M2" t="n">
         <v>2</v>
       </c>
       <c r="N2" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="3">
@@ -554,46 +554,46 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>HABT11</t>
+          <t>TRXF11</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>Multicategoria</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>68.95</v>
+        <v>71.8</v>
       </c>
       <c r="E3" t="n">
-        <v>16.45</v>
+        <v>5.81</v>
       </c>
       <c r="F3" t="n">
-        <v>14.92</v>
+        <v>16.24</v>
       </c>
       <c r="G3" t="n">
-        <v>0.72</v>
+        <v>0.74</v>
       </c>
       <c r="H3" t="n">
-        <v>560342000</v>
+        <v>4482520000</v>
       </c>
       <c r="I3" t="n">
-        <v>1083720</v>
+        <v>40689800</v>
       </c>
       <c r="J3" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
       </c>
       <c r="L3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M3" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="N3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -602,7 +602,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>RPRI11</t>
+          <t>HABT11</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -611,22 +611,22 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>72.37</v>
+        <v>69.95</v>
       </c>
       <c r="E4" t="n">
-        <v>16.99</v>
+        <v>15.34</v>
       </c>
       <c r="F4" t="n">
-        <v>14.73</v>
+        <v>16.05</v>
       </c>
       <c r="G4" t="n">
-        <v>0.72</v>
+        <v>0.75</v>
       </c>
       <c r="H4" t="n">
-        <v>251249000</v>
+        <v>568468000</v>
       </c>
       <c r="I4" t="n">
-        <v>1244300</v>
+        <v>965795</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
@@ -635,10 +635,10 @@
         <v>0</v>
       </c>
       <c r="L4" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="M4" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="N4" t="n">
         <v>9</v>
@@ -650,46 +650,46 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>VCJR11</t>
+          <t>IRIM11</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>Hedge Fund</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>66.91</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="E5" t="n">
+        <v>7.55</v>
+      </c>
+      <c r="F5" t="n">
         <v>15.01</v>
       </c>
-      <c r="F5" t="n">
-        <v>14.46</v>
-      </c>
       <c r="G5" t="n">
-        <v>0.71</v>
+        <v>0.8</v>
       </c>
       <c r="H5" t="n">
-        <v>985181000</v>
+        <v>2321390000</v>
       </c>
       <c r="I5" t="n">
-        <v>2473610</v>
+        <v>3551460</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
       </c>
       <c r="L5" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="M5" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="N5" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6">
@@ -698,46 +698,46 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>IRIM11</t>
+          <t>RZTR11</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Hedge Fund</t>
+          <t>Terras Agrícolas</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>63.25</v>
+        <v>78.5</v>
       </c>
       <c r="E6" t="n">
-        <v>4.02</v>
+        <v>10.46</v>
       </c>
       <c r="F6" t="n">
-        <v>13.66</v>
+        <v>14.48</v>
       </c>
       <c r="G6" t="n">
-        <v>0.75</v>
+        <v>0.8</v>
       </c>
       <c r="H6" t="n">
-        <v>2228040000</v>
+        <v>1479860000</v>
       </c>
       <c r="I6" t="n">
-        <v>2787360</v>
+        <v>3690090</v>
       </c>
       <c r="J6" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
       </c>
       <c r="L6" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="M6" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="N6" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7">
@@ -746,7 +746,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>RBRY11</t>
+          <t>VCJR11</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -755,22 +755,22 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>82.2</v>
+        <v>74.81</v>
       </c>
       <c r="E7" t="n">
-        <v>13.14</v>
+        <v>13.29</v>
       </c>
       <c r="F7" t="n">
-        <v>15.11</v>
+        <v>14.98</v>
       </c>
       <c r="G7" t="n">
         <v>0.8100000000000001</v>
       </c>
       <c r="H7" t="n">
-        <v>1049650000</v>
+        <v>1101500000</v>
       </c>
       <c r="I7" t="n">
-        <v>3691250</v>
+        <v>3482250</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -779,13 +779,13 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="M7" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="N7" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
     </row>
     <row r="8">
@@ -794,46 +794,46 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>RBRX11</t>
+          <t>MCRE11</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Hedge Fund</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>7.38</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="E8" t="n">
-        <v>5.91</v>
+        <v>10.81</v>
       </c>
       <c r="F8" t="n">
-        <v>13.11</v>
+        <v>15.29</v>
       </c>
       <c r="G8" t="n">
-        <v>0.76</v>
+        <v>0.84</v>
       </c>
       <c r="H8" t="n">
-        <v>1080090000</v>
+        <v>936315000</v>
       </c>
       <c r="I8" t="n">
-        <v>2291570</v>
+        <v>3769660</v>
       </c>
       <c r="J8" t="n">
         <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>0</v>
+        <v>11.63</v>
       </c>
       <c r="L8" t="n">
-        <v>7</v>
+        <v>20</v>
       </c>
       <c r="M8" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="N8" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9">
@@ -842,7 +842,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>RVBI11</t>
+          <t>PSEC11</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -851,22 +851,22 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>59.9</v>
+        <v>54</v>
       </c>
       <c r="E9" t="n">
-        <v>13.05</v>
+        <v>12.72</v>
       </c>
       <c r="F9" t="n">
-        <v>14.1</v>
+        <v>13.55</v>
       </c>
       <c r="G9" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.77</v>
       </c>
       <c r="H9" t="n">
-        <v>615533000</v>
+        <v>993566000</v>
       </c>
       <c r="I9" t="n">
-        <v>931734</v>
+        <v>2200470</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
@@ -875,13 +875,13 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="M9" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="N9" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10">
@@ -890,31 +890,31 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>JSAF11</t>
+          <t>RVBI11</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hedge Fund</t>
+          <t>FoF</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>6.86</v>
+        <v>59.9</v>
       </c>
       <c r="E10" t="n">
-        <v>13.68</v>
+        <v>13.05</v>
       </c>
       <c r="F10" t="n">
-        <v>12.76</v>
+        <v>14.1</v>
       </c>
       <c r="G10" t="n">
-        <v>0.74</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="H10" t="n">
-        <v>531810000</v>
+        <v>615533000</v>
       </c>
       <c r="I10" t="n">
-        <v>1510150</v>
+        <v>931734</v>
       </c>
       <c r="J10" t="n">
         <v>0</v>
@@ -923,13 +923,13 @@
         <v>0</v>
       </c>
       <c r="L10" t="n">
-        <v>5</v>
+        <v>14</v>
       </c>
       <c r="M10" t="n">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="N10" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11">
@@ -938,7 +938,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PCIP11</t>
+          <t>RPRI11</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -947,22 +947,22 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>73.76000000000001</v>
+        <v>79.43000000000001</v>
       </c>
       <c r="E11" t="n">
-        <v>13.47</v>
+        <v>15.39</v>
       </c>
       <c r="F11" t="n">
-        <v>12.81</v>
+        <v>13.83</v>
       </c>
       <c r="G11" t="n">
-        <v>0.79</v>
+        <v>0.8</v>
       </c>
       <c r="H11" t="n">
-        <v>1254780000</v>
+        <v>275759000</v>
       </c>
       <c r="I11" t="n">
-        <v>3093400</v>
+        <v>796247</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
@@ -971,13 +971,13 @@
         <v>0</v>
       </c>
       <c r="L11" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="M11" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="N11" t="n">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12">
@@ -986,46 +986,46 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>ITRI11</t>
+          <t>RZAT11</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>FoF</t>
+          <t>Multicategoria</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>73.94</v>
+        <v>87.98</v>
       </c>
       <c r="E12" t="n">
-        <v>14.05</v>
+        <v>12.86</v>
       </c>
       <c r="F12" t="n">
-        <v>12.81</v>
+        <v>15.79</v>
       </c>
       <c r="G12" t="n">
-        <v>0.79</v>
+        <v>0.87</v>
       </c>
       <c r="H12" t="n">
-        <v>462125000</v>
+        <v>372599000</v>
       </c>
       <c r="I12" t="n">
-        <v>1080600</v>
+        <v>544824</v>
       </c>
       <c r="J12" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="M12" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="N12" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13">
@@ -1043,22 +1043,22 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>78.56</v>
+        <v>79.13</v>
       </c>
       <c r="E13" t="n">
-        <v>13.69</v>
+        <v>13.55</v>
       </c>
       <c r="F13" t="n">
-        <v>12.33</v>
+        <v>13.5</v>
       </c>
       <c r="G13" t="n">
-        <v>0.77</v>
+        <v>0.78</v>
       </c>
       <c r="H13" t="n">
-        <v>942720000</v>
+        <v>949560000</v>
       </c>
       <c r="I13" t="n">
-        <v>647629</v>
+        <v>819028</v>
       </c>
       <c r="J13" t="n">
         <v>3</v>
@@ -1067,13 +1067,13 @@
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="M13" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="N13" t="n">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14">
@@ -1082,46 +1082,46 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>VRTA11</t>
+          <t>RBRX11</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>Hedge Fund</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>69.59999999999999</v>
+        <v>7.67</v>
       </c>
       <c r="E14" t="n">
-        <v>14.48</v>
+        <v>7.38</v>
       </c>
       <c r="F14" t="n">
-        <v>13.12</v>
+        <v>13.92</v>
       </c>
       <c r="G14" t="n">
         <v>0.83</v>
       </c>
       <c r="H14" t="n">
-        <v>1085230000</v>
+        <v>1122540000</v>
       </c>
       <c r="I14" t="n">
-        <v>2298850</v>
+        <v>2459870</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="M14" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="N14" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
     </row>
     <row r="15">
@@ -1130,46 +1130,46 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TRXF11</t>
+          <t>RBRR11</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>81.91</v>
+        <v>73.55</v>
       </c>
       <c r="E15" t="n">
-        <v>5.18</v>
+        <v>10.17</v>
       </c>
       <c r="F15" t="n">
-        <v>12.99</v>
+        <v>13.26</v>
       </c>
       <c r="G15" t="n">
-        <v>0.83</v>
+        <v>0.8</v>
       </c>
       <c r="H15" t="n">
-        <v>5113700000</v>
+        <v>1198890000</v>
       </c>
       <c r="I15" t="n">
-        <v>23370000</v>
+        <v>4935700</v>
       </c>
       <c r="J15" t="n">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
       </c>
       <c r="L15" t="n">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="M15" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="N15" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16">
@@ -1178,7 +1178,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HSAF11</t>
+          <t>RZAK11</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1187,22 +1187,22 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>74.89</v>
+        <v>79.44</v>
       </c>
       <c r="E16" t="n">
-        <v>15.02</v>
+        <v>15.01</v>
       </c>
       <c r="F16" t="n">
-        <v>13.61</v>
+        <v>16.01</v>
       </c>
       <c r="G16" t="n">
-        <v>0.84</v>
+        <v>0.9</v>
       </c>
       <c r="H16" t="n">
-        <v>189199000</v>
+        <v>699698000</v>
       </c>
       <c r="I16" t="n">
-        <v>517814</v>
+        <v>1299810</v>
       </c>
       <c r="J16" t="n">
         <v>0</v>
@@ -1211,13 +1211,13 @@
         <v>0</v>
       </c>
       <c r="L16" t="n">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="M16" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="N16" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17">
@@ -1226,7 +1226,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>RZAK11</t>
+          <t>RBRY11</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1235,22 +1235,22 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>77.5</v>
+        <v>88.58</v>
       </c>
       <c r="E17" t="n">
-        <v>13.75</v>
+        <v>11.59</v>
       </c>
       <c r="F17" t="n">
-        <v>15.19</v>
+        <v>14.55</v>
       </c>
       <c r="G17" t="n">
         <v>0.88</v>
       </c>
       <c r="H17" t="n">
-        <v>682611000</v>
+        <v>1131120000</v>
       </c>
       <c r="I17" t="n">
-        <v>1377320</v>
+        <v>4442060</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
@@ -1259,13 +1259,13 @@
         <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="M17" t="n">
-        <v>4</v>
+        <v>14</v>
       </c>
       <c r="N17" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18">
@@ -1274,46 +1274,46 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>MCRE11</t>
+          <t>KISU11</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>FoF</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>8.73</v>
+        <v>6.2</v>
       </c>
       <c r="E18" t="n">
-        <v>10.51</v>
+        <v>9.07</v>
       </c>
       <c r="F18" t="n">
-        <v>13.51</v>
+        <v>13.43</v>
       </c>
       <c r="G18" t="n">
-        <v>0.86</v>
+        <v>0.82</v>
       </c>
       <c r="H18" t="n">
-        <v>974259000</v>
+        <v>369174000</v>
       </c>
       <c r="I18" t="n">
-        <v>2794230</v>
+        <v>652999</v>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" t="n">
-        <v>11.63</v>
+        <v>0</v>
       </c>
       <c r="L18" t="n">
-        <v>31</v>
+        <v>16</v>
       </c>
       <c r="M18" t="n">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="N18" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CPTS11</t>
+          <t>CVBI11</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1331,22 +1331,22 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>7.44</v>
+        <v>82.78</v>
       </c>
       <c r="E19" t="n">
-        <v>6.29</v>
+        <v>14.59</v>
       </c>
       <c r="F19" t="n">
-        <v>12.87</v>
+        <v>14.35</v>
       </c>
       <c r="G19" t="n">
-        <v>0.85</v>
+        <v>0.89</v>
       </c>
       <c r="H19" t="n">
-        <v>2704460000</v>
+        <v>911427000</v>
       </c>
       <c r="I19" t="n">
-        <v>7657600</v>
+        <v>3128870</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
@@ -1355,13 +1355,13 @@
         <v>0</v>
       </c>
       <c r="L19" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="M19" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="N19" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="20">
@@ -1370,7 +1370,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CVBI11</t>
+          <t>VGIP11</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1379,22 +1379,22 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>82.78</v>
+        <v>76.48999999999999</v>
       </c>
       <c r="E20" t="n">
-        <v>14.59</v>
+        <v>11.29</v>
       </c>
       <c r="F20" t="n">
-        <v>14.35</v>
+        <v>13.29</v>
       </c>
       <c r="G20" t="n">
-        <v>0.89</v>
+        <v>0.84</v>
       </c>
       <c r="H20" t="n">
-        <v>911427000</v>
+        <v>901607000</v>
       </c>
       <c r="I20" t="n">
-        <v>3128870</v>
+        <v>1746450</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
@@ -1403,13 +1403,13 @@
         <v>0</v>
       </c>
       <c r="L20" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="M20" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="N20" t="n">
-        <v>56</v>
+        <v>51</v>
       </c>
     </row>
     <row r="21">
@@ -1427,37 +1427,37 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>9.699999999999999</v>
+        <v>10</v>
       </c>
       <c r="E21" t="n">
-        <v>3.43</v>
+        <v>3.81</v>
       </c>
       <c r="F21" t="n">
-        <v>12.4</v>
+        <v>13.54</v>
       </c>
       <c r="G21" t="n">
-        <v>0.84</v>
+        <v>0.87</v>
       </c>
       <c r="H21" t="n">
-        <v>1194690000</v>
+        <v>1231640000</v>
       </c>
       <c r="I21" t="n">
-        <v>5082570</v>
+        <v>3237180</v>
       </c>
       <c r="J21" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="K21" t="n">
-        <v>0</v>
+        <v>6.87</v>
       </c>
       <c r="L21" t="n">
         <v>27</v>
       </c>
       <c r="M21" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="N21" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22">
@@ -1466,43 +1466,43 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>RZTR11</t>
+          <t>BPML11</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Terras Agrícolas</t>
+          <t>Multicategoria</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>84.31999999999999</v>
+        <v>91.13</v>
       </c>
       <c r="E22" t="n">
-        <v>9.880000000000001</v>
+        <v>9.84</v>
       </c>
       <c r="F22" t="n">
-        <v>12.65</v>
+        <v>11.98</v>
       </c>
       <c r="G22" t="n">
-        <v>0.86</v>
+        <v>0.77</v>
       </c>
       <c r="H22" t="n">
-        <v>1589580000</v>
+        <v>678166000</v>
       </c>
       <c r="I22" t="n">
-        <v>2874000</v>
+        <v>1068970</v>
       </c>
       <c r="J22" t="n">
-        <v>29</v>
+        <v>4</v>
       </c>
       <c r="K22" t="n">
-        <v>0</v>
+        <v>7.05</v>
       </c>
       <c r="L22" t="n">
-        <v>31</v>
+        <v>5</v>
       </c>
       <c r="M22" t="n">
-        <v>25</v>
+        <v>51</v>
       </c>
       <c r="N22" t="n">
         <v>56</v>
@@ -1514,46 +1514,46 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>RBRR11</t>
+          <t>TVRI11</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>Escritórios</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>75.44</v>
+        <v>89.97</v>
       </c>
       <c r="E23" t="n">
-        <v>9.199999999999999</v>
+        <v>11.72</v>
       </c>
       <c r="F23" t="n">
-        <v>11.6</v>
+        <v>13.84</v>
       </c>
       <c r="G23" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.9</v>
       </c>
       <c r="H23" t="n">
-        <v>1229690000</v>
+        <v>1432290000</v>
       </c>
       <c r="I23" t="n">
-        <v>4418800</v>
+        <v>967550</v>
       </c>
       <c r="J23" t="n">
-        <v>0</v>
+        <v>57</v>
       </c>
       <c r="K23" t="n">
-        <v>0</v>
+        <v>2.91</v>
       </c>
       <c r="L23" t="n">
-        <v>16</v>
+        <v>38</v>
       </c>
       <c r="M23" t="n">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="N23" t="n">
-        <v>56</v>
+        <v>59</v>
       </c>
     </row>
     <row r="24">
@@ -1562,46 +1562,46 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>TVRI11</t>
+          <t>GGRC11</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Escritórios</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>89.36</v>
+        <v>9.19</v>
       </c>
       <c r="E24" t="n">
-        <v>11.76</v>
+        <v>4.41</v>
       </c>
       <c r="F24" t="n">
-        <v>12.63</v>
+        <v>12.92</v>
       </c>
       <c r="G24" t="n">
-        <v>0.86</v>
+        <v>0.84</v>
       </c>
       <c r="H24" t="n">
-        <v>1422580000</v>
+        <v>3177070000</v>
       </c>
       <c r="I24" t="n">
-        <v>877388</v>
+        <v>15734300</v>
       </c>
       <c r="J24" t="n">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="K24" t="n">
-        <v>5.18</v>
+        <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="M24" t="n">
-        <v>26</v>
+        <v>39</v>
       </c>
       <c r="N24" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
     </row>
     <row r="25">
@@ -1610,7 +1610,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>MANA11</t>
+          <t>JSAF11</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1619,22 +1619,22 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>9.029999999999999</v>
+        <v>7.44</v>
       </c>
       <c r="E25" t="n">
-        <v>10.47</v>
+        <v>13.03</v>
       </c>
       <c r="F25" t="n">
-        <v>26.22</v>
+        <v>12.82</v>
       </c>
       <c r="G25" t="n">
-        <v>0.96</v>
+        <v>0.84</v>
       </c>
       <c r="H25" t="n">
-        <v>338951000</v>
+        <v>576773000</v>
       </c>
       <c r="I25" t="n">
-        <v>1379060</v>
+        <v>1698940</v>
       </c>
       <c r="J25" t="n">
         <v>0</v>
@@ -1643,13 +1643,13 @@
         <v>0</v>
       </c>
       <c r="L25" t="n">
-        <v>56</v>
+        <v>20</v>
       </c>
       <c r="M25" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="N25" t="n">
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="26">
@@ -1667,22 +1667,22 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>8.32</v>
+        <v>8.6</v>
       </c>
       <c r="E26" t="n">
-        <v>13.24</v>
+        <v>13.77</v>
       </c>
       <c r="F26" t="n">
-        <v>12.79</v>
+        <v>13.66</v>
       </c>
       <c r="G26" t="n">
-        <v>0.87</v>
+        <v>0.9</v>
       </c>
       <c r="H26" t="n">
-        <v>310201000</v>
+        <v>320640000</v>
       </c>
       <c r="I26" t="n">
-        <v>624999</v>
+        <v>623744</v>
       </c>
       <c r="J26" t="n">
         <v>0</v>
@@ -1691,13 +1691,13 @@
         <v>0</v>
       </c>
       <c r="L26" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="M26" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="N26" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="27">
@@ -1706,31 +1706,31 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>HFOF11</t>
+          <t>VRTA11</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>FoF</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>6.08</v>
+        <v>75.40000000000001</v>
       </c>
       <c r="E27" t="n">
-        <v>12.52</v>
+        <v>13.84</v>
       </c>
       <c r="F27" t="n">
-        <v>10.33</v>
+        <v>13.37</v>
       </c>
       <c r="G27" t="n">
-        <v>0.78</v>
+        <v>0.89</v>
       </c>
       <c r="H27" t="n">
-        <v>1335730000</v>
+        <v>1175670000</v>
       </c>
       <c r="I27" t="n">
-        <v>2041620</v>
+        <v>1654150</v>
       </c>
       <c r="J27" t="n">
         <v>0</v>
@@ -1739,13 +1739,13 @@
         <v>0</v>
       </c>
       <c r="L27" t="n">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="M27" t="n">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="N27" t="n">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="28">
@@ -1754,31 +1754,31 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>VGIP11</t>
+          <t>XPSF11</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>75.38</v>
+        <v>6.52</v>
       </c>
       <c r="E28" t="n">
-        <v>12.01</v>
+        <v>12.72</v>
       </c>
       <c r="F28" t="n">
-        <v>11.43</v>
+        <v>12.66</v>
       </c>
       <c r="G28" t="n">
-        <v>0.82</v>
+        <v>0.87</v>
       </c>
       <c r="H28" t="n">
-        <v>888523000</v>
+        <v>282330000</v>
       </c>
       <c r="I28" t="n">
-        <v>1956530</v>
+        <v>761393</v>
       </c>
       <c r="J28" t="n">
         <v>0</v>
@@ -1787,13 +1787,13 @@
         <v>0</v>
       </c>
       <c r="L28" t="n">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="M28" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="N28" t="n">
-        <v>64</v>
+        <v>70</v>
       </c>
     </row>
     <row r="29">
@@ -1802,31 +1802,31 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>KFOF11</t>
+          <t>MANA11</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>FoF</t>
+          <t>Hedge Fund</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>75.65000000000001</v>
+        <v>9.23</v>
       </c>
       <c r="E29" t="n">
-        <v>12.41</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="F29" t="n">
-        <v>11.4</v>
+        <v>27.21</v>
       </c>
       <c r="G29" t="n">
-        <v>0.82</v>
+        <v>1</v>
       </c>
       <c r="H29" t="n">
-        <v>530652000</v>
+        <v>346459000</v>
       </c>
       <c r="I29" t="n">
-        <v>1015770</v>
+        <v>1042790</v>
       </c>
       <c r="J29" t="n">
         <v>0</v>
@@ -1835,13 +1835,13 @@
         <v>0</v>
       </c>
       <c r="L29" t="n">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="M29" t="n">
-        <v>45</v>
+        <v>1</v>
       </c>
       <c r="N29" t="n">
-        <v>65</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30">
@@ -1850,46 +1850,46 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>MCLO11</t>
+          <t>VGIR11</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>10.88</v>
+        <v>9.65</v>
       </c>
       <c r="E30" t="n">
-        <v>8.6</v>
+        <v>14.17</v>
       </c>
       <c r="F30" t="n">
-        <v>9.65</v>
+        <v>15.43</v>
       </c>
       <c r="G30" t="n">
-        <v>0.79</v>
+        <v>0.98</v>
       </c>
       <c r="H30" t="n">
-        <v>1356110000</v>
+        <v>1409880000</v>
       </c>
       <c r="I30" t="n">
-        <v>2531740</v>
+        <v>4297540</v>
       </c>
       <c r="J30" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>12</v>
+        <v>63</v>
       </c>
       <c r="M30" t="n">
-        <v>55</v>
+        <v>8</v>
       </c>
       <c r="N30" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="31">
@@ -1898,46 +1898,46 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GGRC11</t>
+          <t>CPTS11</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>9.59</v>
+        <v>7.79</v>
       </c>
       <c r="E31" t="n">
-        <v>5.77</v>
+        <v>5.84</v>
       </c>
       <c r="F31" t="n">
-        <v>12.26</v>
+        <v>13.69</v>
       </c>
       <c r="G31" t="n">
-        <v>0.87</v>
+        <v>0.93</v>
       </c>
       <c r="H31" t="n">
-        <v>2054650000</v>
+        <v>2831690000</v>
       </c>
       <c r="I31" t="n">
-        <v>18370200</v>
+        <v>7272620</v>
       </c>
       <c r="J31" t="n">
-        <v>42</v>
+        <v>0</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
       </c>
       <c r="L31" t="n">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="M31" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="N31" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="32">
@@ -1946,46 +1946,46 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>HSLG11</t>
+          <t>RBVA11</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Varejo</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>84.15000000000001</v>
+        <v>8.93</v>
       </c>
       <c r="E32" t="n">
-        <v>10.85</v>
+        <v>7.37</v>
       </c>
       <c r="F32" t="n">
-        <v>9.19</v>
+        <v>11.97</v>
       </c>
       <c r="G32" t="n">
-        <v>0.77</v>
+        <v>0.84</v>
       </c>
       <c r="H32" t="n">
-        <v>1065340000</v>
+        <v>1475840000</v>
       </c>
       <c r="I32" t="n">
-        <v>14704900</v>
+        <v>1904390</v>
       </c>
       <c r="J32" t="n">
-        <v>6</v>
+        <v>76</v>
       </c>
       <c r="K32" t="n">
-        <v>0</v>
+        <v>4.87</v>
       </c>
       <c r="L32" t="n">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="M32" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="N32" t="n">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="33">
@@ -1994,31 +1994,31 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>VGIR11</t>
+          <t>ITRI11</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>FoF</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>9.56</v>
+        <v>79.2</v>
       </c>
       <c r="E33" t="n">
-        <v>14.81</v>
+        <v>13.32</v>
       </c>
       <c r="F33" t="n">
-        <v>14.38</v>
+        <v>13.03</v>
       </c>
       <c r="G33" t="n">
-        <v>0.98</v>
+        <v>0.9</v>
       </c>
       <c r="H33" t="n">
-        <v>1396730000</v>
+        <v>495000000</v>
       </c>
       <c r="I33" t="n">
-        <v>4223880</v>
+        <v>999663</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
@@ -2027,13 +2027,13 @@
         <v>0</v>
       </c>
       <c r="L33" t="n">
-        <v>60</v>
+        <v>38</v>
       </c>
       <c r="M33" t="n">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="N33" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34">
@@ -2042,46 +2042,46 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>HGRE11</t>
+          <t>PCIP11</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Escritórios</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>114.36</v>
+        <v>81.68000000000001</v>
       </c>
       <c r="E34" t="n">
-        <v>7.71</v>
+        <v>13.74</v>
       </c>
       <c r="F34" t="n">
-        <v>9.17</v>
+        <v>12.57</v>
       </c>
       <c r="G34" t="n">
-        <v>0.78</v>
+        <v>0.88</v>
       </c>
       <c r="H34" t="n">
-        <v>1351480000</v>
+        <v>1389520000</v>
       </c>
       <c r="I34" t="n">
-        <v>2144250</v>
+        <v>3463440</v>
       </c>
       <c r="J34" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K34" t="n">
-        <v>5.93</v>
+        <v>0</v>
       </c>
       <c r="L34" t="n">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="M34" t="n">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="N34" t="n">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="35">
@@ -2090,31 +2090,31 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>BTHF11</t>
+          <t>BTCI11</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Hedge Fund</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>8.699999999999999</v>
+        <v>9.06</v>
       </c>
       <c r="E35" t="n">
-        <v>12.06</v>
+        <v>12.87</v>
       </c>
       <c r="F35" t="n">
-        <v>11.9</v>
+        <v>12.78</v>
       </c>
       <c r="G35" t="n">
-        <v>0.87</v>
+        <v>0.89</v>
       </c>
       <c r="H35" t="n">
-        <v>1790870000</v>
+        <v>901662000</v>
       </c>
       <c r="I35" t="n">
-        <v>3084410</v>
+        <v>3531700</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
@@ -2123,13 +2123,13 @@
         <v>0</v>
       </c>
       <c r="L35" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="M35" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="N35" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="36">
@@ -2138,46 +2138,46 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>RBVA11</t>
+          <t>CLIN11</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Varejo</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>8.880000000000001</v>
+        <v>89.7</v>
       </c>
       <c r="E36" t="n">
-        <v>7.5</v>
+        <v>13.05</v>
       </c>
       <c r="F36" t="n">
-        <v>10.93</v>
+        <v>13.23</v>
       </c>
       <c r="G36" t="n">
-        <v>0.83</v>
+        <v>0.91</v>
       </c>
       <c r="H36" t="n">
-        <v>1386550000</v>
+        <v>389905000</v>
       </c>
       <c r="I36" t="n">
-        <v>2113130</v>
+        <v>1047050</v>
       </c>
       <c r="J36" t="n">
-        <v>74</v>
+        <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>5.97</v>
+        <v>0</v>
       </c>
       <c r="L36" t="n">
-        <v>23</v>
+        <v>42</v>
       </c>
       <c r="M36" t="n">
-        <v>49</v>
+        <v>34</v>
       </c>
       <c r="N36" t="n">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="37">
@@ -2186,7 +2186,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>VILG11</t>
+          <t>HSLG11</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2195,37 +2195,37 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>90.23999999999999</v>
+        <v>86.51000000000001</v>
       </c>
       <c r="E37" t="n">
-        <v>8.94</v>
+        <v>10.87</v>
       </c>
       <c r="F37" t="n">
-        <v>9.279999999999999</v>
+        <v>10.04</v>
       </c>
       <c r="G37" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.79</v>
       </c>
       <c r="H37" t="n">
-        <v>1353360000</v>
+        <v>1095220000</v>
       </c>
       <c r="I37" t="n">
-        <v>2331440</v>
+        <v>1455830</v>
       </c>
       <c r="J37" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="K37" t="n">
-        <v>0.51</v>
+        <v>0</v>
       </c>
       <c r="L37" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="M37" t="n">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="N37" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="38">
@@ -2234,46 +2234,46 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CLIN11</t>
+          <t>TJKB11</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>Hospital</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>86.48</v>
+        <v>256.9</v>
       </c>
       <c r="E38" t="n">
-        <v>13.82</v>
+        <v>6.9</v>
       </c>
       <c r="F38" t="n">
-        <v>11.96</v>
+        <v>13.23</v>
       </c>
       <c r="G38" t="n">
-        <v>0.88</v>
+        <v>0.91</v>
       </c>
       <c r="H38" t="n">
-        <v>375908000</v>
+        <v>548359000</v>
       </c>
       <c r="I38" t="n">
-        <v>649641</v>
+        <v>934859</v>
       </c>
       <c r="J38" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K38" t="n">
         <v>0</v>
       </c>
       <c r="L38" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="M38" t="n">
         <v>34</v>
       </c>
       <c r="N38" t="n">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="39">
@@ -2282,46 +2282,46 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>RZLC11</t>
+          <t>RCRB11</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>Escritórios</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1004.35</v>
+        <v>140</v>
       </c>
       <c r="E39" t="n">
-        <v>6.99</v>
+        <v>6.36</v>
       </c>
       <c r="F39" t="n">
-        <v>14.46</v>
+        <v>9.32</v>
       </c>
       <c r="G39" t="n">
-        <v>1.01</v>
+        <v>0.73</v>
       </c>
       <c r="H39" t="n">
-        <v>162668000</v>
+        <v>516697000</v>
       </c>
       <c r="I39" t="n">
-        <v>940304</v>
+        <v>766836</v>
       </c>
       <c r="J39" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K39" t="n">
         <v>0</v>
       </c>
       <c r="L39" t="n">
-        <v>67</v>
+        <v>2</v>
       </c>
       <c r="M39" t="n">
-        <v>8</v>
+        <v>75</v>
       </c>
       <c r="N39" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40">
@@ -2330,46 +2330,46 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>XPCI11</t>
+          <t>MCLO11</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>78.75</v>
+        <v>10.74</v>
       </c>
       <c r="E40" t="n">
-        <v>16.36</v>
+        <v>8.6</v>
       </c>
       <c r="F40" t="n">
-        <v>12.3</v>
+        <v>9.539999999999999</v>
       </c>
       <c r="G40" t="n">
-        <v>0.89</v>
+        <v>0.78</v>
       </c>
       <c r="H40" t="n">
-        <v>685247000</v>
+        <v>1338660000</v>
       </c>
       <c r="I40" t="n">
-        <v>1610120</v>
+        <v>2231320</v>
       </c>
       <c r="J40" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K40" t="n">
         <v>0</v>
       </c>
       <c r="L40" t="n">
-        <v>45</v>
+        <v>7</v>
       </c>
       <c r="M40" t="n">
-        <v>31</v>
+        <v>72</v>
       </c>
       <c r="N40" t="n">
-        <v>76</v>
+        <v>79</v>
       </c>
     </row>
     <row r="41">
@@ -2378,46 +2378,46 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ICRI11</t>
+          <t>SNEL11</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>89.95</v>
+        <v>7.97</v>
       </c>
       <c r="E41" t="n">
-        <v>14.18</v>
+        <v>4.44</v>
       </c>
       <c r="F41" t="n">
-        <v>11.78</v>
+        <v>14.87</v>
       </c>
       <c r="G41" t="n">
-        <v>0.88</v>
+        <v>0.99</v>
       </c>
       <c r="H41" t="n">
-        <v>346969000</v>
+        <v>1809580000</v>
       </c>
       <c r="I41" t="n">
-        <v>635554</v>
+        <v>8593590</v>
       </c>
       <c r="J41" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K41" t="n">
         <v>0</v>
       </c>
       <c r="L41" t="n">
-        <v>39</v>
+        <v>66</v>
       </c>
       <c r="M41" t="n">
-        <v>38</v>
+        <v>13</v>
       </c>
       <c r="N41" t="n">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="42">
@@ -2426,46 +2426,46 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>TRXB11</t>
+          <t>NEWL11</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Renda Urbana</t>
+          <t>Multicategoria</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>185.92</v>
+        <v>110.4</v>
       </c>
       <c r="E42" t="n">
-        <v>4.58</v>
+        <v>13.89</v>
       </c>
       <c r="F42" t="n">
-        <v>17.93</v>
+        <v>10.75</v>
       </c>
       <c r="G42" t="n">
-        <v>1.88</v>
+        <v>0.84</v>
       </c>
       <c r="H42" t="n">
-        <v>755955000</v>
+        <v>310245000</v>
       </c>
       <c r="I42" t="n">
-        <v>658545</v>
+        <v>560495</v>
       </c>
       <c r="J42" t="n">
-        <v>11</v>
+        <v>2</v>
       </c>
       <c r="K42" t="n">
         <v>0</v>
       </c>
       <c r="L42" t="n">
-        <v>74</v>
+        <v>20</v>
       </c>
       <c r="M42" t="n">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="N42" t="n">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="43">
@@ -2474,46 +2474,46 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>AZPL11</t>
+          <t>BTHF11</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Hedge Fund</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>7.38</v>
+        <v>8.94</v>
       </c>
       <c r="E43" t="n">
-        <v>8.83</v>
+        <v>11.74</v>
       </c>
       <c r="F43" t="n">
-        <v>11.09</v>
+        <v>13.25</v>
       </c>
       <c r="G43" t="n">
-        <v>0.86</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H43" t="n">
-        <v>309389000</v>
+        <v>1840270000</v>
       </c>
       <c r="I43" t="n">
-        <v>889732</v>
+        <v>4072150</v>
       </c>
       <c r="J43" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="M43" t="n">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="N43" t="n">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="44">
@@ -2522,46 +2522,46 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>BTCI11</t>
+          <t>IBBP11</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>8.99</v>
+        <v>8</v>
       </c>
       <c r="E44" t="n">
-        <v>12.85</v>
+        <v>7.86</v>
       </c>
       <c r="F44" t="n">
-        <v>11.47</v>
+        <v>11.71</v>
       </c>
       <c r="G44" t="n">
         <v>0.88</v>
       </c>
       <c r="H44" t="n">
-        <v>894695000</v>
+        <v>602965000</v>
       </c>
       <c r="I44" t="n">
-        <v>4890560</v>
+        <v>889841</v>
       </c>
       <c r="J44" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="K44" t="n">
-        <v>0</v>
+        <v>0.23</v>
       </c>
       <c r="L44" t="n">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="M44" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="N44" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="45">
@@ -2570,46 +2570,46 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PMLL11</t>
+          <t>ICRI11</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Shoppings</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>100.5</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="E45" t="n">
-        <v>10.35</v>
+        <v>13.19</v>
       </c>
       <c r="F45" t="n">
-        <v>10.05</v>
+        <v>12.95</v>
       </c>
       <c r="G45" t="n">
-        <v>0.86</v>
+        <v>0.93</v>
       </c>
       <c r="H45" t="n">
-        <v>1405200000</v>
+        <v>359120000</v>
       </c>
       <c r="I45" t="n">
-        <v>4621910</v>
+        <v>738299</v>
       </c>
       <c r="J45" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="K45" t="n">
-        <v>3.69</v>
+        <v>0</v>
       </c>
       <c r="L45" t="n">
-        <v>31</v>
+        <v>48</v>
       </c>
       <c r="M45" t="n">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="N45" t="n">
-        <v>83</v>
+        <v>86</v>
       </c>
     </row>
     <row r="46">
@@ -2618,46 +2618,46 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>XPLG11</t>
+          <t>TRXB11</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Renda Urbana</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>89.91</v>
+        <v>192.12</v>
       </c>
       <c r="E46" t="n">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="F46" t="n">
-        <v>9.859999999999999</v>
+        <v>16.96</v>
       </c>
       <c r="G46" t="n">
-        <v>0.85</v>
+        <v>1.88</v>
       </c>
       <c r="H46" t="n">
-        <v>4620480000</v>
+        <v>781164000</v>
       </c>
       <c r="I46" t="n">
-        <v>8978070</v>
+        <v>7374700</v>
       </c>
       <c r="J46" t="n">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="K46" t="n">
-        <v>9.34</v>
+        <v>0</v>
       </c>
       <c r="L46" t="n">
-        <v>29</v>
+        <v>84</v>
       </c>
       <c r="M46" t="n">
-        <v>54</v>
+        <v>3</v>
       </c>
       <c r="N46" t="n">
-        <v>83</v>
+        <v>87</v>
       </c>
     </row>
     <row r="47">
@@ -2666,46 +2666,46 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>KNHF11</t>
+          <t>CPLG11</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Hedge Fund</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>90.76000000000001</v>
+        <v>11</v>
       </c>
       <c r="E47" t="n">
-        <v>14.11</v>
+        <v>1.79</v>
       </c>
       <c r="F47" t="n">
-        <v>11.86</v>
+        <v>15.35</v>
       </c>
       <c r="G47" t="n">
-        <v>0.9</v>
+        <v>1.02</v>
       </c>
       <c r="H47" t="n">
-        <v>1784640000</v>
+        <v>619913000</v>
       </c>
       <c r="I47" t="n">
-        <v>3382020</v>
+        <v>2249360</v>
       </c>
       <c r="J47" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K47" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="L47" t="n">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="M47" t="n">
-        <v>36</v>
+        <v>9</v>
       </c>
       <c r="N47" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
     <row r="48">
@@ -2714,31 +2714,31 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>HGCR11</t>
+          <t>HFOF11</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>FoF</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>89.67</v>
+        <v>6.53</v>
       </c>
       <c r="E48" t="n">
-        <v>12.39</v>
+        <v>11.69</v>
       </c>
       <c r="F48" t="n">
-        <v>11.79</v>
+        <v>10.74</v>
       </c>
       <c r="G48" t="n">
-        <v>0.91</v>
+        <v>0.87</v>
       </c>
       <c r="H48" t="n">
-        <v>1382540000</v>
+        <v>1422100000</v>
       </c>
       <c r="I48" t="n">
-        <v>3138790</v>
+        <v>1590160</v>
       </c>
       <c r="J48" t="n">
         <v>0</v>
@@ -2747,13 +2747,13 @@
         <v>0</v>
       </c>
       <c r="L48" t="n">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="M48" t="n">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="N48" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
     </row>
     <row r="49">
@@ -2762,46 +2762,46 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>GARE11</t>
+          <t>XPCI11</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>8.16</v>
+        <v>82.45</v>
       </c>
       <c r="E49" t="n">
-        <v>5.25</v>
+        <v>15.83</v>
       </c>
       <c r="F49" t="n">
-        <v>10.96</v>
+        <v>12.82</v>
       </c>
       <c r="G49" t="n">
-        <v>0.88</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H49" t="n">
-        <v>2359760000</v>
+        <v>717443000</v>
       </c>
       <c r="I49" t="n">
-        <v>10103400</v>
+        <v>1708520</v>
       </c>
       <c r="J49" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
       </c>
       <c r="L49" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="M49" t="n">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="N49" t="n">
-        <v>87</v>
+        <v>90</v>
       </c>
     </row>
     <row r="50">
@@ -2810,46 +2810,46 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>FATN11</t>
+          <t>RZLC11</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Escritórios</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>77.90000000000001</v>
+        <v>1006.08</v>
       </c>
       <c r="E50" t="n">
-        <v>5.38</v>
+        <v>9.390000000000001</v>
       </c>
       <c r="F50" t="n">
-        <v>7.98</v>
+        <v>14.35</v>
       </c>
       <c r="G50" t="n">
-        <v>0.8</v>
+        <v>1.01</v>
       </c>
       <c r="H50" t="n">
-        <v>526469000</v>
+        <v>162948000</v>
       </c>
       <c r="I50" t="n">
-        <v>2327470</v>
+        <v>1554390</v>
       </c>
       <c r="J50" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="K50" t="n">
-        <v>20.92</v>
+        <v>0</v>
       </c>
       <c r="L50" t="n">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="M50" t="n">
-        <v>73</v>
+        <v>16</v>
       </c>
       <c r="N50" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="51">
@@ -2858,46 +2858,46 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>MALL11</t>
+          <t>FATN11</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Shoppings</t>
+          <t>Escritórios</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>100.03</v>
+        <v>86.90000000000001</v>
       </c>
       <c r="E51" t="n">
-        <v>14.22</v>
+        <v>6.22</v>
       </c>
       <c r="F51" t="n">
-        <v>8.91</v>
+        <v>10.94</v>
       </c>
       <c r="G51" t="n">
-        <v>0.83</v>
+        <v>0.89</v>
       </c>
       <c r="H51" t="n">
-        <v>1398630000</v>
+        <v>614378000</v>
       </c>
       <c r="I51" t="n">
-        <v>1520130</v>
+        <v>1641850</v>
       </c>
       <c r="J51" t="n">
-        <v>11</v>
+        <v>63</v>
       </c>
       <c r="K51" t="n">
-        <v>3.64</v>
+        <v>23.47</v>
       </c>
       <c r="L51" t="n">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="M51" t="n">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="N51" t="n">
-        <v>88</v>
+        <v>92</v>
       </c>
     </row>
     <row r="52">
@@ -2906,46 +2906,46 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>SNEL11</t>
+          <t>KNUQ11</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>8.359999999999999</v>
+        <v>101.79</v>
       </c>
       <c r="E52" t="n">
-        <v>5.74</v>
+        <v>13.68</v>
       </c>
       <c r="F52" t="n">
-        <v>12.85</v>
+        <v>14.03</v>
       </c>
       <c r="G52" t="n">
-        <v>1.05</v>
+        <v>1.01</v>
       </c>
       <c r="H52" t="n">
-        <v>925118000</v>
+        <v>2186930000</v>
       </c>
       <c r="I52" t="n">
-        <v>6874160</v>
+        <v>5585030</v>
       </c>
       <c r="J52" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K52" t="n">
         <v>0</v>
       </c>
       <c r="L52" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="M52" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="N52" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="53">
@@ -2954,46 +2954,46 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>LVBI11</t>
+          <t>HGRE11</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Escritórios</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>99.34999999999999</v>
+        <v>124.79</v>
       </c>
       <c r="E53" t="n">
-        <v>9.02</v>
+        <v>7.21</v>
       </c>
       <c r="F53" t="n">
-        <v>8.18</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="G53" t="n">
-        <v>0.82</v>
+        <v>0.83</v>
       </c>
       <c r="H53" t="n">
-        <v>1601380000</v>
+        <v>1474740000</v>
       </c>
       <c r="I53" t="n">
-        <v>3192610</v>
+        <v>2467650</v>
       </c>
       <c r="J53" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="K53" t="n">
-        <v>5.75</v>
+        <v>5.93</v>
       </c>
       <c r="L53" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="M53" t="n">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="N53" t="n">
-        <v>91</v>
+        <v>94</v>
       </c>
     </row>
     <row r="54">
@@ -3002,46 +3002,46 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MXRF11</t>
+          <t>MALL11</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>Shoppings</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>9.35</v>
+        <v>100.03</v>
       </c>
       <c r="E54" t="n">
-        <v>11.23</v>
+        <v>14.22</v>
       </c>
       <c r="F54" t="n">
-        <v>12.52</v>
+        <v>8.91</v>
       </c>
       <c r="G54" t="n">
-        <v>1</v>
+        <v>0.83</v>
       </c>
       <c r="H54" t="n">
-        <v>4303520000</v>
+        <v>1398630000</v>
       </c>
       <c r="I54" t="n">
-        <v>15001600</v>
+        <v>1520130</v>
       </c>
       <c r="J54" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K54" t="n">
-        <v>0</v>
+        <v>3.64</v>
       </c>
       <c r="L54" t="n">
-        <v>65</v>
+        <v>17</v>
       </c>
       <c r="M54" t="n">
-        <v>28</v>
+        <v>78</v>
       </c>
       <c r="N54" t="n">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="55">
@@ -3050,46 +3050,46 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>RINV11</t>
+          <t>MXRF11</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>101.25</v>
+        <v>9.34</v>
       </c>
       <c r="E55" t="n">
-        <v>8.779999999999999</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="F55" t="n">
-        <v>11.62</v>
+        <v>13.7</v>
       </c>
       <c r="G55" t="n">
-        <v>0.95</v>
+        <v>1.01</v>
       </c>
       <c r="H55" t="n">
-        <v>509457000</v>
+        <v>5297710000</v>
       </c>
       <c r="I55" t="n">
-        <v>549888</v>
+        <v>25041400</v>
       </c>
       <c r="J55" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K55" t="n">
         <v>0</v>
       </c>
       <c r="L55" t="n">
-        <v>55</v>
+        <v>74</v>
       </c>
       <c r="M55" t="n">
-        <v>39</v>
+        <v>23</v>
       </c>
       <c r="N55" t="n">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="56">
@@ -3098,31 +3098,31 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>KNUQ11</t>
+          <t>KFOF11</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>FoF</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>104.14</v>
+        <v>81.83</v>
       </c>
       <c r="E56" t="n">
-        <v>12.33</v>
+        <v>11.22</v>
       </c>
       <c r="F56" t="n">
-        <v>12.62</v>
+        <v>11.61</v>
       </c>
       <c r="G56" t="n">
-        <v>1.03</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="H56" t="n">
-        <v>2237420000</v>
+        <v>574002000</v>
       </c>
       <c r="I56" t="n">
-        <v>4129240</v>
+        <v>1017800</v>
       </c>
       <c r="J56" t="n">
         <v>0</v>
@@ -3131,13 +3131,13 @@
         <v>0</v>
       </c>
       <c r="L56" t="n">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="M56" t="n">
-        <v>27</v>
+        <v>55</v>
       </c>
       <c r="N56" t="n">
-        <v>96</v>
+        <v>105</v>
       </c>
     </row>
     <row r="57">
@@ -3146,46 +3146,46 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>MCCI11</t>
+          <t>LVBI11</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>93</v>
+        <v>102.45</v>
       </c>
       <c r="E57" t="n">
-        <v>11.53</v>
+        <v>8.81</v>
       </c>
       <c r="F57" t="n">
-        <v>11.57</v>
+        <v>8.81</v>
       </c>
       <c r="G57" t="n">
-        <v>0.98</v>
+        <v>0.85</v>
       </c>
       <c r="H57" t="n">
-        <v>1577280000</v>
+        <v>1651350000</v>
       </c>
       <c r="I57" t="n">
-        <v>5012850</v>
+        <v>4453970</v>
       </c>
       <c r="J57" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="K57" t="n">
-        <v>0</v>
+        <v>3.02</v>
       </c>
       <c r="L57" t="n">
-        <v>60</v>
+        <v>26</v>
       </c>
       <c r="M57" t="n">
-        <v>41</v>
+        <v>79</v>
       </c>
       <c r="N57" t="n">
-        <v>101</v>
+        <v>105</v>
       </c>
     </row>
     <row r="58">
@@ -3194,31 +3194,31 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>KNCR11</t>
+          <t>KNHF11</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>Hedge Fund</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>105.6</v>
+        <v>95.75</v>
       </c>
       <c r="E58" t="n">
-        <v>9.93</v>
+        <v>14.44</v>
       </c>
       <c r="F58" t="n">
-        <v>12.1</v>
+        <v>12.39</v>
       </c>
       <c r="G58" t="n">
-        <v>1.03</v>
+        <v>0.97</v>
       </c>
       <c r="H58" t="n">
-        <v>11308700000</v>
+        <v>1882750000</v>
       </c>
       <c r="I58" t="n">
-        <v>20928500</v>
+        <v>5607370</v>
       </c>
       <c r="J58" t="n">
         <v>0</v>
@@ -3227,13 +3227,13 @@
         <v>0</v>
       </c>
       <c r="L58" t="n">
-        <v>69</v>
+        <v>58</v>
       </c>
       <c r="M58" t="n">
-        <v>33</v>
+        <v>48</v>
       </c>
       <c r="N58" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="59">
@@ -3242,46 +3242,46 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>AFHI11</t>
+          <t>PMLL11</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Papel</t>
+          <t>Shoppings</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>94</v>
+        <v>108.99</v>
       </c>
       <c r="E59" t="n">
-        <v>11.59</v>
+        <v>7.62</v>
       </c>
       <c r="F59" t="n">
-        <v>11.48</v>
+        <v>10.52</v>
       </c>
       <c r="G59" t="n">
-        <v>0.99</v>
+        <v>0.91</v>
       </c>
       <c r="H59" t="n">
-        <v>450184000</v>
+        <v>1934620000</v>
       </c>
       <c r="I59" t="n">
-        <v>713635</v>
+        <v>3266680</v>
       </c>
       <c r="J59" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="K59" t="n">
-        <v>0</v>
+        <v>4.07</v>
       </c>
       <c r="L59" t="n">
-        <v>63</v>
+        <v>42</v>
       </c>
       <c r="M59" t="n">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="N59" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
     </row>
     <row r="60">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>KNIP11</t>
+          <t>GARE11</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -3299,37 +3299,37 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>89.40000000000001</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="E60" t="n">
-        <v>12.94</v>
+        <v>7.7</v>
       </c>
       <c r="F60" t="n">
-        <v>10.09</v>
+        <v>11.44</v>
       </c>
       <c r="G60" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="H60" t="n">
-        <v>7158990000</v>
+        <v>2492790000</v>
       </c>
       <c r="I60" t="n">
-        <v>10781300</v>
+        <v>6678480</v>
       </c>
       <c r="J60" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K60" t="n">
         <v>0</v>
       </c>
       <c r="L60" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="M60" t="n">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="N60" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="61">
@@ -3338,46 +3338,46 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>HGRU11</t>
+          <t>HGBS11</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Renda Urbana</t>
+          <t>Shoppings</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>116.8</v>
+        <v>19.27</v>
       </c>
       <c r="E61" t="n">
-        <v>8.52</v>
+        <v>8.23</v>
       </c>
       <c r="F61" t="n">
-        <v>9.220000000000001</v>
+        <v>10.13</v>
       </c>
       <c r="G61" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="H61" t="n">
-        <v>2714200000</v>
+        <v>2781730000</v>
       </c>
       <c r="I61" t="n">
-        <v>6286520</v>
+        <v>7133270</v>
       </c>
       <c r="J61" t="n">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="K61" t="n">
-        <v>0.8100000000000001</v>
+        <v>4.28</v>
       </c>
       <c r="L61" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="M61" t="n">
-        <v>58</v>
+        <v>66</v>
       </c>
       <c r="N61" t="n">
-        <v>107</v>
+        <v>112</v>
       </c>
     </row>
     <row r="62">
@@ -3386,46 +3386,46 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>HGLG11</t>
+          <t>RBRL11</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>145.55</v>
+        <v>85.06</v>
       </c>
       <c r="E62" t="n">
-        <v>6.68</v>
+        <v>8.6</v>
       </c>
       <c r="F62" t="n">
-        <v>8.19</v>
+        <v>9.44</v>
       </c>
       <c r="G62" t="n">
-        <v>0.88</v>
+        <v>0.91</v>
       </c>
       <c r="H62" t="n">
-        <v>6637330000</v>
+        <v>568799000</v>
       </c>
       <c r="I62" t="n">
-        <v>17266200</v>
+        <v>1359810</v>
       </c>
       <c r="J62" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="K62" t="n">
-        <v>3.23</v>
+        <v>0</v>
       </c>
       <c r="L62" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="M62" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="N62" t="n">
-        <v>109</v>
+        <v>115</v>
       </c>
     </row>
     <row r="63">
@@ -3434,46 +3434,46 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>HGBS11</t>
+          <t>KNCR11</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Shoppings</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>18.81</v>
+        <v>105.66</v>
       </c>
       <c r="E63" t="n">
-        <v>8.130000000000001</v>
+        <v>10.72</v>
       </c>
       <c r="F63" t="n">
-        <v>9.199999999999999</v>
+        <v>13.01</v>
       </c>
       <c r="G63" t="n">
-        <v>0.92</v>
+        <v>1.03</v>
       </c>
       <c r="H63" t="n">
-        <v>2715330000</v>
+        <v>11315100000</v>
       </c>
       <c r="I63" t="n">
-        <v>4397500</v>
+        <v>25961800</v>
       </c>
       <c r="J63" t="n">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c r="K63" t="n">
-        <v>4.31</v>
+        <v>0</v>
       </c>
       <c r="L63" t="n">
-        <v>51</v>
+        <v>80</v>
       </c>
       <c r="M63" t="n">
-        <v>59</v>
+        <v>37</v>
       </c>
       <c r="N63" t="n">
-        <v>110</v>
+        <v>117</v>
       </c>
     </row>
     <row r="64">
@@ -3482,46 +3482,46 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>VISC11</t>
+          <t>BTRU11</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Shoppings</t>
+          <t>Outros</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>103.24</v>
+        <v>83.34999999999999</v>
       </c>
       <c r="E64" t="n">
-        <v>5.88</v>
+        <v>7.86</v>
       </c>
       <c r="F64" t="n">
-        <v>8.66</v>
+        <v>11.46</v>
       </c>
       <c r="G64" t="n">
-        <v>0.89</v>
+        <v>0.98</v>
       </c>
       <c r="H64" t="n">
-        <v>2976270000</v>
+        <v>741709000</v>
       </c>
       <c r="I64" t="n">
-        <v>4675760</v>
+        <v>10534000</v>
       </c>
       <c r="J64" t="n">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="K64" t="n">
-        <v>5.74</v>
+        <v>0</v>
       </c>
       <c r="L64" t="n">
-        <v>45</v>
+        <v>63</v>
       </c>
       <c r="M64" t="n">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="N64" t="n">
-        <v>112</v>
+        <v>119</v>
       </c>
     </row>
     <row r="65">
@@ -3530,46 +3530,46 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ALZR11</t>
+          <t>HGCR11</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>9.869999999999999</v>
+        <v>97.89</v>
       </c>
       <c r="E65" t="n">
-        <v>7.69</v>
+        <v>10.94</v>
       </c>
       <c r="F65" t="n">
-        <v>9.16</v>
+        <v>11.82</v>
       </c>
       <c r="G65" t="n">
-        <v>0.92</v>
+        <v>0.99</v>
       </c>
       <c r="H65" t="n">
-        <v>1623740000</v>
+        <v>1509280000</v>
       </c>
       <c r="I65" t="n">
-        <v>3107340</v>
+        <v>3523320</v>
       </c>
       <c r="J65" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="K65" t="n">
-        <v>12.46</v>
+        <v>0</v>
       </c>
       <c r="L65" t="n">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="M65" t="n">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="N65" t="n">
-        <v>113</v>
+        <v>119</v>
       </c>
     </row>
     <row r="66">
@@ -3578,31 +3578,31 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>KNSC11</t>
+          <t>MCCI11</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>8.960000000000001</v>
+        <v>94.90000000000001</v>
       </c>
       <c r="E66" t="n">
-        <v>13.76</v>
+        <v>10.86</v>
       </c>
       <c r="F66" t="n">
-        <v>11.31</v>
+        <v>12.5</v>
       </c>
       <c r="G66" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="H66" t="n">
-        <v>1811730000</v>
+        <v>1609510000</v>
       </c>
       <c r="I66" t="n">
-        <v>4200810</v>
+        <v>6151280</v>
       </c>
       <c r="J66" t="n">
         <v>0</v>
@@ -3611,13 +3611,13 @@
         <v>0</v>
       </c>
       <c r="L66" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="M66" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N66" t="n">
-        <v>114</v>
+        <v>119</v>
       </c>
     </row>
     <row r="67">
@@ -3626,46 +3626,46 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>HSRE11</t>
+          <t>KNHY11</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Renda Urbana</t>
+          <t>Multicategoria</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>86.45</v>
+        <v>99.12</v>
       </c>
       <c r="E67" t="n">
-        <v>7.39</v>
+        <v>12.52</v>
       </c>
       <c r="F67" t="n">
-        <v>10.04</v>
+        <v>12.35</v>
       </c>
       <c r="G67" t="n">
         <v>1</v>
       </c>
       <c r="H67" t="n">
-        <v>769295000</v>
+        <v>3089880000</v>
       </c>
       <c r="I67" t="n">
-        <v>3770130</v>
+        <v>5339520</v>
       </c>
       <c r="J67" t="n">
-        <v>22</v>
+        <v>0</v>
       </c>
       <c r="K67" t="n">
         <v>0</v>
       </c>
       <c r="L67" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="M67" t="n">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="N67" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="68">
@@ -3674,46 +3674,46 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>KNHY11</t>
+          <t>VILG11</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>97.68000000000001</v>
+        <v>100.5</v>
       </c>
       <c r="E68" t="n">
-        <v>12.27</v>
+        <v>8.31</v>
       </c>
       <c r="F68" t="n">
-        <v>9.58</v>
+        <v>9.41</v>
       </c>
       <c r="G68" t="n">
-        <v>0.99</v>
+        <v>0.92</v>
       </c>
       <c r="H68" t="n">
-        <v>3044990000</v>
+        <v>1507240000</v>
       </c>
       <c r="I68" t="n">
-        <v>3842470</v>
+        <v>3703240</v>
       </c>
       <c r="J68" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="K68" t="n">
-        <v>0</v>
+        <v>0.44</v>
       </c>
       <c r="L68" t="n">
-        <v>63</v>
+        <v>46</v>
       </c>
       <c r="M68" t="n">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="N68" t="n">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="69">
@@ -3722,7 +3722,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>HPDP11</t>
+          <t>XPML11</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -3731,37 +3731,37 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>87.98999999999999</v>
+        <v>105.99</v>
       </c>
       <c r="E69" t="n">
-        <v>4.34</v>
+        <v>8.69</v>
       </c>
       <c r="F69" t="n">
-        <v>8.109999999999999</v>
+        <v>10.32</v>
       </c>
       <c r="G69" t="n">
-        <v>0.92</v>
+        <v>0.96</v>
       </c>
       <c r="H69" t="n">
-        <v>620417000</v>
+        <v>6816010000</v>
       </c>
       <c r="I69" t="n">
-        <v>828346</v>
+        <v>23414800</v>
       </c>
       <c r="J69" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="K69" t="n">
-        <v>1.65</v>
+        <v>5.2</v>
       </c>
       <c r="L69" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="M69" t="n">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="N69" t="n">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="70">
@@ -3770,46 +3770,46 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>BRCO11</t>
+          <t>AFHI11</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Logística</t>
+          <t>Papel</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>111.9</v>
+        <v>96</v>
       </c>
       <c r="E70" t="n">
-        <v>7.28</v>
+        <v>10.26</v>
       </c>
       <c r="F70" t="n">
-        <v>8.800000000000001</v>
+        <v>12.4</v>
       </c>
       <c r="G70" t="n">
-        <v>0.97</v>
+        <v>1.01</v>
       </c>
       <c r="H70" t="n">
-        <v>2016580000</v>
+        <v>507726000</v>
       </c>
       <c r="I70" t="n">
-        <v>4908510</v>
+        <v>902325</v>
       </c>
       <c r="J70" t="n">
-        <v>14</v>
+        <v>0</v>
       </c>
       <c r="K70" t="n">
-        <v>12.62</v>
+        <v>0</v>
       </c>
       <c r="L70" t="n">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="M70" t="n">
-        <v>66</v>
+        <v>47</v>
       </c>
       <c r="N70" t="n">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="71">
@@ -3818,46 +3818,46 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>PQDP11</t>
+          <t>PQAG11</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Shoppings</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>2514.96</v>
+        <v>54.53</v>
       </c>
       <c r="E71" t="n">
-        <v>5.19</v>
+        <v>10.73</v>
       </c>
       <c r="F71" t="n">
-        <v>8.25</v>
+        <v>10.61</v>
       </c>
       <c r="G71" t="n">
         <v>0.97</v>
       </c>
       <c r="H71" t="n">
-        <v>614186000</v>
+        <v>762978000</v>
       </c>
       <c r="I71" t="n">
-        <v>2085960</v>
+        <v>1463520</v>
       </c>
       <c r="J71" t="n">
         <v>1</v>
       </c>
       <c r="K71" t="n">
-        <v>0.66</v>
+        <v>0</v>
       </c>
       <c r="L71" t="n">
         <v>58</v>
       </c>
       <c r="M71" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="N71" t="n">
-        <v>127</v>
+        <v>121</v>
       </c>
     </row>
     <row r="72">
@@ -3866,46 +3866,46 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>KNRI11</t>
+          <t>XPLG11</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>152.18</v>
+        <v>99.89</v>
       </c>
       <c r="E72" t="n">
-        <v>7.58</v>
+        <v>7.39</v>
       </c>
       <c r="F72" t="n">
-        <v>7.71</v>
+        <v>9.76</v>
       </c>
       <c r="G72" t="n">
-        <v>0.93</v>
+        <v>0.95</v>
       </c>
       <c r="H72" t="n">
-        <v>4292090000</v>
+        <v>5133360000</v>
       </c>
       <c r="I72" t="n">
-        <v>7483780</v>
+        <v>9398730</v>
       </c>
       <c r="J72" t="n">
-        <v>18</v>
+        <v>30</v>
       </c>
       <c r="K72" t="n">
-        <v>0.09</v>
+        <v>16.5</v>
       </c>
       <c r="L72" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M72" t="n">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="N72" t="n">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="73">
@@ -3914,46 +3914,46 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>BTLG11</t>
+          <t>BRCO11</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Multicategoria</t>
+          <t>Logística</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>100.38</v>
+        <v>111.5</v>
       </c>
       <c r="E73" t="n">
-        <v>6</v>
+        <v>7.44</v>
       </c>
       <c r="F73" t="n">
-        <v>8.57</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="G73" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="H73" t="n">
-        <v>6965330000</v>
+        <v>2009380000</v>
       </c>
       <c r="I73" t="n">
-        <v>11570200</v>
+        <v>8038760</v>
       </c>
       <c r="J73" t="n">
-        <v>31</v>
+        <v>14</v>
       </c>
       <c r="K73" t="n">
-        <v>5.06</v>
+        <v>9.529999999999999</v>
       </c>
       <c r="L73" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="M73" t="n">
         <v>68</v>
       </c>
       <c r="N73" t="n">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="74">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>CPUR11</t>
+          <t>KNIP11</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -3971,37 +3971,37 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>10.97</v>
+        <v>92.51000000000001</v>
       </c>
       <c r="E74" t="n">
-        <v>6.87</v>
+        <v>13.41</v>
       </c>
       <c r="F74" t="n">
-        <v>9.050000000000001</v>
+        <v>10.81</v>
       </c>
       <c r="G74" t="n">
-        <v>1.13</v>
+        <v>0.99</v>
       </c>
       <c r="H74" t="n">
-        <v>744048000</v>
+        <v>7408030000</v>
       </c>
       <c r="I74" t="n">
-        <v>13844800</v>
+        <v>9997040</v>
       </c>
       <c r="J74" t="n">
-        <v>18</v>
+        <v>0</v>
       </c>
       <c r="K74" t="n">
-        <v>0.62</v>
+        <v>0</v>
       </c>
       <c r="L74" t="n">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="M74" t="n">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="N74" t="n">
-        <v>135</v>
+        <v>126</v>
       </c>
     </row>
     <row r="75">
@@ -4010,46 +4010,526 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>HBCR11</t>
+          <t>HGRU11</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
+          <t>Renda Urbana</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>123.38</v>
+      </c>
+      <c r="E75" t="n">
+        <v>7.26</v>
+      </c>
+      <c r="F75" t="n">
+        <v>9.56</v>
+      </c>
+      <c r="G75" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="H75" t="n">
+        <v>3064040000</v>
+      </c>
+      <c r="I75" t="n">
+        <v>9800550</v>
+      </c>
+      <c r="J75" t="n">
+        <v>98</v>
+      </c>
+      <c r="K75" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="L75" t="n">
+        <v>56</v>
+      </c>
+      <c r="M75" t="n">
+        <v>71</v>
+      </c>
+      <c r="N75" t="n">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ALZR11</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
           <t>Multicategoria</t>
         </is>
       </c>
-      <c r="D75" t="n">
-        <v>153.52</v>
-      </c>
-      <c r="E75" t="n">
-        <v>5.13</v>
-      </c>
-      <c r="F75" t="n">
-        <v>8.94</v>
-      </c>
-      <c r="G75" t="n">
-        <v>1.31</v>
-      </c>
-      <c r="H75" t="n">
-        <v>245632000</v>
-      </c>
-      <c r="I75" t="n">
-        <v>8768020</v>
-      </c>
-      <c r="J75" t="n">
-        <v>3</v>
-      </c>
-      <c r="K75" t="n">
-        <v>0</v>
-      </c>
-      <c r="L75" t="n">
-        <v>73</v>
-      </c>
-      <c r="M75" t="n">
-        <v>64</v>
-      </c>
-      <c r="N75" t="n">
-        <v>137</v>
+      <c r="D76" t="n">
+        <v>10.41</v>
+      </c>
+      <c r="E76" t="n">
+        <v>8.119999999999999</v>
+      </c>
+      <c r="F76" t="n">
+        <v>9.57</v>
+      </c>
+      <c r="G76" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="H76" t="n">
+        <v>1711410000</v>
+      </c>
+      <c r="I76" t="n">
+        <v>5656180</v>
+      </c>
+      <c r="J76" t="n">
+        <v>20</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0</v>
+      </c>
+      <c r="L76" t="n">
+        <v>58</v>
+      </c>
+      <c r="M76" t="n">
+        <v>70</v>
+      </c>
+      <c r="N76" t="n">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>RINV11</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Multicategoria</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>106.8</v>
+      </c>
+      <c r="E77" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F77" t="n">
+        <v>12.47</v>
+      </c>
+      <c r="G77" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="H77" t="n">
+        <v>537383000</v>
+      </c>
+      <c r="I77" t="n">
+        <v>555758</v>
+      </c>
+      <c r="J77" t="n">
+        <v>0</v>
+      </c>
+      <c r="K77" t="n">
+        <v>0</v>
+      </c>
+      <c r="L77" t="n">
+        <v>83</v>
+      </c>
+      <c r="M77" t="n">
+        <v>46</v>
+      </c>
+      <c r="N77" t="n">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>KNSC11</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Multicategoria</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>9.16</v>
+      </c>
+      <c r="E78" t="n">
+        <v>13.93</v>
+      </c>
+      <c r="F78" t="n">
+        <v>12.18</v>
+      </c>
+      <c r="G78" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="H78" t="n">
+        <v>1870060000</v>
+      </c>
+      <c r="I78" t="n">
+        <v>5669300</v>
+      </c>
+      <c r="J78" t="n">
+        <v>0</v>
+      </c>
+      <c r="K78" t="n">
+        <v>0</v>
+      </c>
+      <c r="L78" t="n">
+        <v>81</v>
+      </c>
+      <c r="M78" t="n">
+        <v>50</v>
+      </c>
+      <c r="N78" t="n">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>BTLG11</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Multicategoria</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>102.5</v>
+      </c>
+      <c r="E79" t="n">
+        <v>6.41</v>
+      </c>
+      <c r="F79" t="n">
+        <v>9.32</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="H79" t="n">
+        <v>7271380000</v>
+      </c>
+      <c r="I79" t="n">
+        <v>23322400</v>
+      </c>
+      <c r="J79" t="n">
+        <v>30</v>
+      </c>
+      <c r="K79" t="n">
+        <v>2.16</v>
+      </c>
+      <c r="L79" t="n">
+        <v>58</v>
+      </c>
+      <c r="M79" t="n">
+        <v>75</v>
+      </c>
+      <c r="N79" t="n">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>HGLG11</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Multicategoria</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>156.42</v>
+      </c>
+      <c r="E80" t="n">
+        <v>7.12</v>
+      </c>
+      <c r="F80" t="n">
+        <v>8.51</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="H80" t="n">
+        <v>7133020000</v>
+      </c>
+      <c r="I80" t="n">
+        <v>22771900</v>
+      </c>
+      <c r="J80" t="n">
+        <v>37</v>
+      </c>
+      <c r="K80" t="n">
+        <v>2.41</v>
+      </c>
+      <c r="L80" t="n">
+        <v>53</v>
+      </c>
+      <c r="M80" t="n">
+        <v>81</v>
+      </c>
+      <c r="N80" t="n">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>CPUR11</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Multicategoria</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>10.43</v>
+      </c>
+      <c r="E81" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="F81" t="n">
+        <v>10.84</v>
+      </c>
+      <c r="G81" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="H81" t="n">
+        <v>707423000</v>
+      </c>
+      <c r="I81" t="n">
+        <v>4167840</v>
+      </c>
+      <c r="J81" t="n">
+        <v>14</v>
+      </c>
+      <c r="K81" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="L81" t="n">
+        <v>81</v>
+      </c>
+      <c r="M81" t="n">
+        <v>59</v>
+      </c>
+      <c r="N81" t="n">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>VISC11</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Shoppings</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>113.6</v>
+      </c>
+      <c r="E82" t="n">
+        <v>6.04</v>
+      </c>
+      <c r="F82" t="n">
+        <v>8.720000000000001</v>
+      </c>
+      <c r="G82" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="H82" t="n">
+        <v>3274930000</v>
+      </c>
+      <c r="I82" t="n">
+        <v>8449500</v>
+      </c>
+      <c r="J82" t="n">
+        <v>32</v>
+      </c>
+      <c r="K82" t="n">
+        <v>5.78</v>
+      </c>
+      <c r="L82" t="n">
+        <v>63</v>
+      </c>
+      <c r="M82" t="n">
+        <v>80</v>
+      </c>
+      <c r="N82" t="n">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>KNRI11</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Multicategoria</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>161.95</v>
+      </c>
+      <c r="E83" t="n">
+        <v>6.85</v>
+      </c>
+      <c r="F83" t="n">
+        <v>8.1</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="H83" t="n">
+        <v>4567650000</v>
+      </c>
+      <c r="I83" t="n">
+        <v>7919430</v>
+      </c>
+      <c r="J83" t="n">
+        <v>18</v>
+      </c>
+      <c r="K83" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="L83" t="n">
+        <v>66</v>
+      </c>
+      <c r="M83" t="n">
+        <v>84</v>
+      </c>
+      <c r="N83" t="n">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>PQDP11</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Shoppings</t>
+        </is>
+      </c>
+      <c r="D84" t="n">
+        <v>2590</v>
+      </c>
+      <c r="E84" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="F84" t="n">
+        <v>8.49</v>
+      </c>
+      <c r="G84" t="n">
+        <v>1</v>
+      </c>
+      <c r="H84" t="n">
+        <v>671079000</v>
+      </c>
+      <c r="I84" t="n">
+        <v>7506690</v>
+      </c>
+      <c r="J84" t="n">
+        <v>1</v>
+      </c>
+      <c r="K84" t="n">
+        <v>0</v>
+      </c>
+      <c r="L84" t="n">
+        <v>70</v>
+      </c>
+      <c r="M84" t="n">
+        <v>82</v>
+      </c>
+      <c r="N84" t="n">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>HIRE11</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Outros</t>
+        </is>
+      </c>
+      <c r="D85" t="n">
+        <v>100.36</v>
+      </c>
+      <c r="E85" t="n">
+        <v>5.63</v>
+      </c>
+      <c r="F85" t="n">
+        <v>8.210000000000001</v>
+      </c>
+      <c r="G85" t="n">
+        <v>1</v>
+      </c>
+      <c r="H85" t="n">
+        <v>275017000</v>
+      </c>
+      <c r="I85" t="n">
+        <v>4197370</v>
+      </c>
+      <c r="J85" t="n">
+        <v>4</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0</v>
+      </c>
+      <c r="L85" t="n">
+        <v>70</v>
+      </c>
+      <c r="M85" t="n">
+        <v>83</v>
+      </c>
+      <c r="N85" t="n">
+        <v>153</v>
       </c>
     </row>
   </sheetData>

</xml_diff>